<commit_message>
uodate annoation xlsx add SPARQL column
</commit_message>
<xml_diff>
--- a/Annotation/annotation_outputs/annotation_group_1.xlsx
+++ b/Annotation/annotation_outputs/annotation_group_1.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$K$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Sheet1'!$A$1:$M$100</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -497,20 +497,22 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K100"/>
+  <dimension ref="A1:M100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
     <col width="45" customWidth="1" min="2" max="2"/>
     <col width="35" customWidth="1" min="3" max="3"/>
     <col width="35" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="24" customWidth="1" min="6" max="6"/>
-    <col width="24" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
-    <col width="45" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="12" max="12"/>
+    <col width="45" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -536,35 +538,45 @@
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
+          <t>SPARQL</t>
+        </is>
+      </c>
+      <c r="F1" s="3" t="inlineStr">
+        <is>
+          <t>Corrected SPARQL</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
           <t>taxonomy_label</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>source</t>
         </is>
       </c>
-      <c r="G1" s="3" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>label_correctness</t>
         </is>
       </c>
-      <c r="H1" s="3" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>missing_edge</t>
         </is>
       </c>
-      <c r="I1" s="3" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>missing_node</t>
         </is>
       </c>
-      <c r="J1" s="3" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>missing_property_or_qualifier</t>
         </is>
       </c>
-      <c r="K1" s="3" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>note</t>
         </is>
@@ -591,19 +603,33 @@
       </c>
       <c r="E2" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?movie ?label WHERE {
+  ?movie wdt:P31 wd:Q11424 .
+  ?movie rdfs:label ?label .
+  ?movie wdt:P577 ?release .
+  FILTER(LANG(?label) = "en")
+  FILTER(CONTAINS(LCASE(?label) , "planet of the apes"))
+}
+GROUP BY ?movie ?label
+ORDER BY MIN(?release)</t>
+        </is>
+      </c>
+      <c r="F2" s="5" t="inlineStr"/>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00603.json</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr"/>
-      <c r="H2" s="5" t="inlineStr"/>
       <c r="I2" s="5" t="inlineStr"/>
       <c r="J2" s="5" t="inlineStr"/>
       <c r="K2" s="5" t="inlineStr"/>
+      <c r="L2" s="5" t="inlineStr"/>
+      <c r="M2" s="5" t="inlineStr"/>
     </row>
     <row r="3" ht="65" customHeight="1">
       <c r="A3" s="6" t="n">
@@ -626,19 +652,34 @@
       </c>
       <c r="E3" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?president ?presidentLabel WHERE {
+  wd:Q1580241 wdt:P571 ?start ; wdt:P576 ?end .
+  ?president p:P39 ?statement .
+  ?statement ps:P39 wd:Q11696 .
+  ?statement pq:P580 ?termStart ; pq:P582 ?termEnd .
+  FILTER(?termStart &lt;= ?end &amp;&amp; ?termEnd &gt;= ?start)
+  .
+  ?president rdfs:label ?presidentLabel .
+  FILTER(LANG(?presidentLabel) = "en")
+}</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr"/>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F3" s="6" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_infobox_complex/00076.json</t>
         </is>
       </c>
-      <c r="G3" s="7" t="inlineStr"/>
-      <c r="H3" s="7" t="inlineStr"/>
       <c r="I3" s="7" t="inlineStr"/>
       <c r="J3" s="7" t="inlineStr"/>
       <c r="K3" s="7" t="inlineStr"/>
+      <c r="L3" s="7" t="inlineStr"/>
+      <c r="M3" s="7" t="inlineStr"/>
     </row>
     <row r="4" ht="65" customHeight="1">
       <c r="A4" s="4" t="n">
@@ -661,19 +702,29 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?award ?awardLabel WHERE {
+  wd:Q451558 wdt:P166 ?award .
+  ?award rdfs:label ?awardLabel .
+  FILTER(LANG(?awardLabel) = "en")
+}</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr"/>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F4" s="4" t="inlineStr">
+      <c r="H4" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00143.json</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr"/>
-      <c r="H4" s="5" t="inlineStr"/>
       <c r="I4" s="5" t="inlineStr"/>
       <c r="J4" s="5" t="inlineStr"/>
       <c r="K4" s="5" t="inlineStr"/>
+      <c r="L4" s="5" t="inlineStr"/>
+      <c r="M4" s="5" t="inlineStr"/>
     </row>
     <row r="5" ht="65" customHeight="1">
       <c r="A5" s="6" t="n">
@@ -696,19 +747,34 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?award ?awardLabel WHERE {
+  wd:Q26505 p:P166 ?statement .
+  ?statement ps:P166 ?award .
+  ?statement pq:P585 ?time .
+  FILTER(YEAR(?time) = 1953)
+  OPTIONAL {
+    ?award rdfs:label ?awardLabel
+    FILTER(LANG(?awardLabel) = "en")
+  }
+}</t>
+        </is>
+      </c>
+      <c r="F5" s="7" t="inlineStr"/>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_infobox_complex/00035.json</t>
         </is>
       </c>
-      <c r="G5" s="7" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr"/>
       <c r="I5" s="7" t="inlineStr"/>
       <c r="J5" s="7" t="inlineStr"/>
       <c r="K5" s="7" t="inlineStr"/>
+      <c r="L5" s="7" t="inlineStr"/>
+      <c r="M5" s="7" t="inlineStr"/>
     </row>
     <row r="6" ht="65" customHeight="1">
       <c r="A6" s="4" t="n">
@@ -731,19 +797,31 @@
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?country ?countryLabel WHERE {
+  wd:Q7176 wdt:P166 wd:Q95919064 .
+  wd:Q95919064 wdt:P361 ?order .
+  ?order wdt:P17 ?country .
+  ?country rdfs:label ?countryLabel
+  FILTER(lang(?countryLabel) = "en")
+}</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr"/>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F6" s="4" t="inlineStr">
+      <c r="H6" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00280.json</t>
         </is>
       </c>
-      <c r="G6" s="5" t="inlineStr"/>
-      <c r="H6" s="5" t="inlineStr"/>
       <c r="I6" s="5" t="inlineStr"/>
       <c r="J6" s="5" t="inlineStr"/>
       <c r="K6" s="5" t="inlineStr"/>
+      <c r="L6" s="5" t="inlineStr"/>
+      <c r="M6" s="5" t="inlineStr"/>
     </row>
     <row r="7" ht="65" customHeight="1">
       <c r="A7" s="6" t="n">
@@ -766,19 +844,29 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?genreLabel WHERE {
+  wd:Q3268056 wdt:P136 ?genre .
+  ?genre rdfs:label ?genreLabel .
+  FILTER(LANG(?genreLabel) = "en")
+}</t>
+        </is>
+      </c>
+      <c r="F7" s="7" t="inlineStr"/>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00522.json</t>
         </is>
       </c>
-      <c r="G7" s="7" t="inlineStr"/>
-      <c r="H7" s="7" t="inlineStr"/>
       <c r="I7" s="7" t="inlineStr"/>
       <c r="J7" s="7" t="inlineStr"/>
       <c r="K7" s="7" t="inlineStr"/>
+      <c r="L7" s="7" t="inlineStr"/>
+      <c r="M7" s="7" t="inlineStr"/>
     </row>
     <row r="8" ht="65" customHeight="1">
       <c r="A8" s="4" t="n">
@@ -801,19 +889,31 @@
       </c>
       <c r="E8" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?network ?networkLabel WHERE {
+  wd:Q1088765 wdt:P449 ?network .
+  OPTIONAL {
+    ?network rdfs:label ?networkLabel
+    FILTER(lang(?networkLabel) = "en")
+  }
+}</t>
+        </is>
+      </c>
+      <c r="F8" s="5" t="inlineStr"/>
+      <c r="G8" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F8" s="4" t="inlineStr">
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00278.json</t>
         </is>
       </c>
-      <c r="G8" s="5" t="inlineStr"/>
-      <c r="H8" s="5" t="inlineStr"/>
       <c r="I8" s="5" t="inlineStr"/>
       <c r="J8" s="5" t="inlineStr"/>
       <c r="K8" s="5" t="inlineStr"/>
+      <c r="L8" s="5" t="inlineStr"/>
+      <c r="M8" s="5" t="inlineStr"/>
     </row>
     <row r="9" ht="65" customHeight="1">
       <c r="A9" s="6" t="n">
@@ -836,19 +936,30 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?country ?countryLabel WHERE {
+  wd:Q39444 wdt:P54 / wdt:P17 ?country .
+  ?country rdfs:label ?countryLabel .
+  FILTER(LANG(?countryLabel) = "en")
+}
+GROUP BY ?country ?countryLabel</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr"/>
+      <c r="G9" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00148.json</t>
         </is>
       </c>
-      <c r="G9" s="7" t="inlineStr"/>
-      <c r="H9" s="7" t="inlineStr"/>
       <c r="I9" s="7" t="inlineStr"/>
       <c r="J9" s="7" t="inlineStr"/>
       <c r="K9" s="7" t="inlineStr"/>
+      <c r="L9" s="7" t="inlineStr"/>
+      <c r="M9" s="7" t="inlineStr"/>
     </row>
     <row r="10" ht="65" customHeight="1">
       <c r="A10" s="4" t="n">
@@ -871,19 +982,36 @@
       </c>
       <c r="E10" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?composer ?composerLabel ?performer ?performerLabel WHERE {
+  wd:Q5976590 wdt:P86 ?composer .
+  wd:Q5976590 wdt:P175 ?performer .
+  OPTIONAL {
+    ?composer rdfs:label ?composerLabel
+    FILTER(LANG(?composerLabel) = "en")
+  }
+  OPTIONAL {
+    ?performer rdfs:label ?performerLabel
+    FILTER(LANG(?performerLabel) = "en")
+  }
+}</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr"/>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F10" s="4" t="inlineStr">
+      <c r="H10" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00682.json</t>
         </is>
       </c>
-      <c r="G10" s="5" t="inlineStr"/>
-      <c r="H10" s="5" t="inlineStr"/>
       <c r="I10" s="5" t="inlineStr"/>
       <c r="J10" s="5" t="inlineStr"/>
       <c r="K10" s="5" t="inlineStr"/>
+      <c r="L10" s="5" t="inlineStr"/>
+      <c r="M10" s="5" t="inlineStr"/>
     </row>
     <row r="11" ht="65" customHeight="1">
       <c r="A11" s="6" t="n">
@@ -906,19 +1034,30 @@
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?screenwriter ?name WHERE {
+  wd:Q161087 wdt:P58 ?screenwriter .
+  ?screenwriter rdfs:label ?name .
+  FILTER(LANG(?name) = "en")
+  .
+}</t>
+        </is>
+      </c>
+      <c r="F11" s="7" t="inlineStr"/>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_table_complex/00027.json</t>
         </is>
       </c>
-      <c r="G11" s="7" t="inlineStr"/>
-      <c r="H11" s="7" t="inlineStr"/>
       <c r="I11" s="7" t="inlineStr"/>
       <c r="J11" s="7" t="inlineStr"/>
       <c r="K11" s="7" t="inlineStr"/>
+      <c r="L11" s="7" t="inlineStr"/>
+      <c r="M11" s="7" t="inlineStr"/>
     </row>
     <row r="12" ht="65" customHeight="1">
       <c r="A12" s="4" t="n">
@@ -941,19 +1080,31 @@
       </c>
       <c r="E12" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?singer ?label WHERE {
+  ?singer wdt:P463 wd:Q126826 .
+  ?singer wdt:P106 wd:Q177220 .
+  ?singer rdfs:label ?label .
+  FILTER(LANG(?label) = 'en')
+  .
+}</t>
+        </is>
+      </c>
+      <c r="F12" s="5" t="inlineStr"/>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F12" s="4" t="inlineStr">
+      <c r="H12" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_infobox_complex/00130.json</t>
         </is>
       </c>
-      <c r="G12" s="5" t="inlineStr"/>
-      <c r="H12" s="5" t="inlineStr"/>
       <c r="I12" s="5" t="inlineStr"/>
       <c r="J12" s="5" t="inlineStr"/>
       <c r="K12" s="5" t="inlineStr"/>
+      <c r="L12" s="5" t="inlineStr"/>
+      <c r="M12" s="5" t="inlineStr"/>
     </row>
     <row r="13" ht="65" customHeight="1">
       <c r="A13" s="6" t="n">
@@ -976,19 +1127,27 @@
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?date WHERE {
+  wd:Q155476 wdt:P577 ?date .
+}</t>
+        </is>
+      </c>
+      <c r="F13" s="7" t="inlineStr"/>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F13" s="6" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00962.json</t>
         </is>
       </c>
-      <c r="G13" s="7" t="inlineStr"/>
-      <c r="H13" s="7" t="inlineStr"/>
       <c r="I13" s="7" t="inlineStr"/>
       <c r="J13" s="7" t="inlineStr"/>
       <c r="K13" s="7" t="inlineStr"/>
+      <c r="L13" s="7" t="inlineStr"/>
+      <c r="M13" s="7" t="inlineStr"/>
     </row>
     <row r="14" ht="65" customHeight="1">
       <c r="A14" s="4" t="n">
@@ -1011,19 +1170,45 @@
       </c>
       <c r="E14" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?film ?filmLabel(COUNT(?award) AS ?count) WHERE {
+  {
+    ?film wdt:P57 wd:Q43203
+  } UNION {
+    ?film wdt:P162 wd:Q43203
+  }
+  ?film wdt:P31 wd:Q11424 .
+  ?film wdt:P166 ?award .
+  {
+    ?award wdt:P31 wd:Q19020
+  } UNION {
+    ?award wdt:P179 wd:Q335485
+  }
+  OPTIONAL {
+    ?film rdfs:label ?filmLabel .
+    FILTER(LANG(?filmLabel) = "en")
+  }
+}
+GROUP BY ?film ?filmLabel
+ORDER BY DESC(?count)
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F14" s="5" t="inlineStr"/>
+      <c r="G14" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F14" s="4" t="inlineStr">
+      <c r="H14" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_table_complex/00053.json</t>
         </is>
       </c>
-      <c r="G14" s="5" t="inlineStr"/>
-      <c r="H14" s="5" t="inlineStr"/>
       <c r="I14" s="5" t="inlineStr"/>
       <c r="J14" s="5" t="inlineStr"/>
       <c r="K14" s="5" t="inlineStr"/>
+      <c r="L14" s="5" t="inlineStr"/>
+      <c r="M14" s="5" t="inlineStr"/>
     </row>
     <row r="15" ht="65" customHeight="1">
       <c r="A15" s="6" t="n">
@@ -1046,19 +1231,27 @@
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?inception WHERE {
+  wd:Q2636724 wdt:P571 ?inception
+}</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr"/>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00281.json</t>
         </is>
       </c>
-      <c r="G15" s="7" t="inlineStr"/>
-      <c r="H15" s="7" t="inlineStr"/>
       <c r="I15" s="7" t="inlineStr"/>
       <c r="J15" s="7" t="inlineStr"/>
       <c r="K15" s="7" t="inlineStr"/>
+      <c r="L15" s="7" t="inlineStr"/>
+      <c r="M15" s="7" t="inlineStr"/>
     </row>
     <row r="16" ht="65" customHeight="1">
       <c r="A16" s="4" t="n">
@@ -1081,19 +1274,30 @@
       </c>
       <c r="E16" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?team(YEAR(?end) - YEAR(?start) AS ?duration) WHERE {
+  wd:Q184269 p:P54 ?statement .
+  ?statement ps:P54 ?team ; pq:P580 ?start ; pq:P582 ?end .
+}
+ORDER BY DESC(?duration)
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr"/>
+      <c r="G16" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F16" s="4" t="inlineStr">
+      <c r="H16" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_table_complex/00187.json</t>
         </is>
       </c>
-      <c r="G16" s="5" t="inlineStr"/>
-      <c r="H16" s="5" t="inlineStr"/>
       <c r="I16" s="5" t="inlineStr"/>
       <c r="J16" s="5" t="inlineStr"/>
       <c r="K16" s="5" t="inlineStr"/>
+      <c r="L16" s="5" t="inlineStr"/>
+      <c r="M16" s="5" t="inlineStr"/>
     </row>
     <row r="17" ht="65" customHeight="1">
       <c r="A17" s="6" t="n">
@@ -1116,19 +1320,35 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?book ?date WHERE {
+  {
+    wd:Q752584 wdt:P577 ?date .
+    BIND(wd:Q752584 AS ?book)
+  } UNION {
+    wd:Q478016 wdt:P577 ?date .
+    BIND(wd:Q478016 AS ?book)
+  }
+}
+ORDER BY ?date
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F17" s="7" t="inlineStr"/>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_infobox_complex/00295.json</t>
         </is>
       </c>
-      <c r="G17" s="7" t="inlineStr"/>
-      <c r="H17" s="7" t="inlineStr"/>
       <c r="I17" s="7" t="inlineStr"/>
       <c r="J17" s="7" t="inlineStr"/>
       <c r="K17" s="7" t="inlineStr"/>
+      <c r="L17" s="7" t="inlineStr"/>
+      <c r="M17" s="7" t="inlineStr"/>
     </row>
     <row r="18" ht="65" customHeight="1">
       <c r="A18" s="4" t="n">
@@ -1151,19 +1371,27 @@
       </c>
       <c r="E18" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?author WHERE {
+  wd:Q127912 wdt:P50 ?author .
+}</t>
+        </is>
+      </c>
+      <c r="F18" s="5" t="inlineStr"/>
+      <c r="G18" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F18" s="4" t="inlineStr">
+      <c r="H18" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00312.json</t>
         </is>
       </c>
-      <c r="G18" s="5" t="inlineStr"/>
-      <c r="H18" s="5" t="inlineStr"/>
       <c r="I18" s="5" t="inlineStr"/>
       <c r="J18" s="5" t="inlineStr"/>
       <c r="K18" s="5" t="inlineStr"/>
+      <c r="L18" s="5" t="inlineStr"/>
+      <c r="M18" s="5" t="inlineStr"/>
     </row>
     <row r="19" ht="65" customHeight="1">
       <c r="A19" s="6" t="n">
@@ -1186,19 +1414,30 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?actor ?label WHERE {
+  wd:Q957323 wdt:P161 ?actor .
+  wd:Q651923 wdt:P161 ?actor .
+  ?actor rdfs:label ?label .
+  FILTER(LANG(?label) = "en")
+}</t>
+        </is>
+      </c>
+      <c r="F19" s="7" t="inlineStr"/>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F19" s="6" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_infobox_complex/00024.json</t>
         </is>
       </c>
-      <c r="G19" s="7" t="inlineStr"/>
-      <c r="H19" s="7" t="inlineStr"/>
       <c r="I19" s="7" t="inlineStr"/>
       <c r="J19" s="7" t="inlineStr"/>
       <c r="K19" s="7" t="inlineStr"/>
+      <c r="L19" s="7" t="inlineStr"/>
+      <c r="M19" s="7" t="inlineStr"/>
     </row>
     <row r="20" ht="65" customHeight="1">
       <c r="A20" s="4" t="n">
@@ -1221,19 +1460,40 @@
       </c>
       <c r="E20" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?recipientLabel ?languageLabel WHERE {
+  {
+    SELECT ?recipient WHERE {
+      ?recipient p:P166 ?stmt .
+      ?stmt ps:P166 wd:Q916783 .
+      ?stmt pq:P585 ?time .
+    }
+    ORDER BY ASC(?time)
+    LIMIT 1
+  }
+  ?recipient wdt:P1412 ?language .
+  ?recipient rdfs:label ?recipientLabel .
+  ?language rdfs:label ?languageLabel .
+  FILTER(LANG(?recipientLabel) = 'en')
+  FILTER(LANG(?languageLabel) = 'en')
+}</t>
+        </is>
+      </c>
+      <c r="F20" s="5" t="inlineStr"/>
+      <c r="G20" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F20" s="4" t="inlineStr">
+      <c r="H20" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00258.json</t>
         </is>
       </c>
-      <c r="G20" s="5" t="inlineStr"/>
-      <c r="H20" s="5" t="inlineStr"/>
       <c r="I20" s="5" t="inlineStr"/>
       <c r="J20" s="5" t="inlineStr"/>
       <c r="K20" s="5" t="inlineStr"/>
+      <c r="L20" s="5" t="inlineStr"/>
+      <c r="M20" s="5" t="inlineStr"/>
     </row>
     <row r="21" ht="65" customHeight="1">
       <c r="A21" s="6" t="n">
@@ -1256,19 +1516,33 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?team ?teamLabel(COUNT(*) AS ?wins) WHERE {
+  ?cupFinal wdt:P31 wd:Q211872 .
+  ?cupFinal wdt:P1346 ?team .
+  ?team rdfs:label ?teamLabel .
+  FILTER(LANG(?teamLabel) = "en")
+}
+GROUP BY ?team ?teamLabel
+ORDER BY DESC(?wins)
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F21" s="7" t="inlineStr"/>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F21" s="6" t="inlineStr">
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00011.json</t>
         </is>
       </c>
-      <c r="G21" s="7" t="inlineStr"/>
-      <c r="H21" s="7" t="inlineStr"/>
       <c r="I21" s="7" t="inlineStr"/>
       <c r="J21" s="7" t="inlineStr"/>
       <c r="K21" s="7" t="inlineStr"/>
+      <c r="L21" s="7" t="inlineStr"/>
+      <c r="M21" s="7" t="inlineStr"/>
     </row>
     <row r="22" ht="65" customHeight="1">
       <c r="A22" s="4" t="n">
@@ -1291,19 +1565,27 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?singer WHERE {
+  wd:Q27000439 wdt:P175 ?singer .
+}</t>
+        </is>
+      </c>
+      <c r="F22" s="5" t="inlineStr"/>
+      <c r="G22" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F22" s="4" t="inlineStr">
+      <c r="H22" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00129.json</t>
         </is>
       </c>
-      <c r="G22" s="5" t="inlineStr"/>
-      <c r="H22" s="5" t="inlineStr"/>
       <c r="I22" s="5" t="inlineStr"/>
       <c r="J22" s="5" t="inlineStr"/>
       <c r="K22" s="5" t="inlineStr"/>
+      <c r="L22" s="5" t="inlineStr"/>
+      <c r="M22" s="5" t="inlineStr"/>
     </row>
     <row r="23" ht="65" customHeight="1">
       <c r="A23" s="6" t="n">
@@ -1326,19 +1608,32 @@
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?book ?bookLabel ?publicationDate WHERE {
+  wd:Q96277193 wdt:P527 ?book .
+  ?book wdt:P577 ?publicationDate .
+  ?book rdfs:label ?bookLabel .
+  FILTER(LANG(?bookLabel) = 'en')
+}
+ORDER BY DESC(?publicationDate)
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F23" s="7" t="inlineStr"/>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F23" s="6" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_table_complex/00091.json</t>
         </is>
       </c>
-      <c r="G23" s="7" t="inlineStr"/>
-      <c r="H23" s="7" t="inlineStr"/>
       <c r="I23" s="7" t="inlineStr"/>
       <c r="J23" s="7" t="inlineStr"/>
       <c r="K23" s="7" t="inlineStr"/>
+      <c r="L23" s="7" t="inlineStr"/>
+      <c r="M23" s="7" t="inlineStr"/>
     </row>
     <row r="24" ht="65" customHeight="1">
       <c r="A24" s="4" t="n">
@@ -1361,19 +1656,34 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?country ?countryLabel(COUNT(?medal) AS ?medalCount) WHERE {
+  ?athlete wdt:P1344 wd:Q9678 .
+  ?athlete wdt:P166 ?medal .
+  ?athlete wdt:P27 ?country .
+  ?country rdfs:label ?countryLabel .
+  FILTER(LANG(?countryLabel) = "en")
+}
+GROUP BY ?country ?countryLabel
+ORDER BY DESC(?medalCount)
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr"/>
+      <c r="G24" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F24" s="4" t="inlineStr">
+      <c r="H24" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00113.json</t>
         </is>
       </c>
-      <c r="G24" s="5" t="inlineStr"/>
-      <c r="H24" s="5" t="inlineStr"/>
       <c r="I24" s="5" t="inlineStr"/>
       <c r="J24" s="5" t="inlineStr"/>
       <c r="K24" s="5" t="inlineStr"/>
+      <c r="L24" s="5" t="inlineStr"/>
+      <c r="M24" s="5" t="inlineStr"/>
     </row>
     <row r="25" ht="65" customHeight="1">
       <c r="A25" s="6" t="n">
@@ -1396,19 +1706,36 @@
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?movie ?movieLabel(MIN(?boxOffice) AS ?minBoxOffice) WHERE {
+  ?movie wdt:P31 wd:Q11424 .
+  ?movie rdfs:label ?movieLabel .
+  ?movie wdt:P2142 ?boxOffice .
+  FILTER(LANG(?movieLabel) = 'en')
+  .
+  FILTER CONTAINS(LCASE(?movieLabel) , 'terminator')
+}
+GROUP BY ?movie ?movieLabel
+HAVING(COUNT(?boxOffice) &gt;= 1)
+ORDER BY ASC(?minBoxOffice)
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F25" s="7" t="inlineStr"/>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F25" s="6" t="inlineStr">
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_table_complex/00261.json</t>
         </is>
       </c>
-      <c r="G25" s="7" t="inlineStr"/>
-      <c r="H25" s="7" t="inlineStr"/>
       <c r="I25" s="7" t="inlineStr"/>
       <c r="J25" s="7" t="inlineStr"/>
       <c r="K25" s="7" t="inlineStr"/>
+      <c r="L25" s="7" t="inlineStr"/>
+      <c r="M25" s="7" t="inlineStr"/>
     </row>
     <row r="26" ht="65" customHeight="1">
       <c r="A26" s="4" t="n">
@@ -1431,19 +1758,32 @@
       </c>
       <c r="E26" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?sponsor ?sponsorLabel WHERE {
+  wd:Q20855983 wdt:P859 ?sponsor .
+  OPTIONAL {
+    ?sponsor rdfs:label ?sponsorLabel
+    FILTER(LANG(?sponsorLabel) = "en")
+    .
+  }
+}</t>
+        </is>
+      </c>
+      <c r="F26" s="5" t="inlineStr"/>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F26" s="4" t="inlineStr">
+      <c r="H26" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00214.json</t>
         </is>
       </c>
-      <c r="G26" s="5" t="inlineStr"/>
-      <c r="H26" s="5" t="inlineStr"/>
       <c r="I26" s="5" t="inlineStr"/>
       <c r="J26" s="5" t="inlineStr"/>
       <c r="K26" s="5" t="inlineStr"/>
+      <c r="L26" s="5" t="inlineStr"/>
+      <c r="M26" s="5" t="inlineStr"/>
     </row>
     <row r="27" ht="65" customHeight="1">
       <c r="A27" s="6" t="n">
@@ -1466,19 +1806,36 @@
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?movie ?movieLabel ?collection WHERE {
+  wd:Q162255 wdt:P179 ?series .
+  ?movie wdt:P179 ?series .
+  ?movie wdt:P31 / wdt:P279 * wd:Q11424 .
+  ?movie wdt:P2142 ?collection .
+  OPTIONAL {
+    ?movie rdfs:label ?movieLabel .
+    FILTER(LANG(?movieLabel) = "en")
+  }
+}
+ORDER BY DESC(xsd:decimal(?collection))
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F27" s="7" t="inlineStr"/>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F27" s="6" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_table_complex/00248.json</t>
         </is>
       </c>
-      <c r="G27" s="7" t="inlineStr"/>
-      <c r="H27" s="7" t="inlineStr"/>
       <c r="I27" s="7" t="inlineStr"/>
       <c r="J27" s="7" t="inlineStr"/>
       <c r="K27" s="7" t="inlineStr"/>
+      <c r="L27" s="7" t="inlineStr"/>
+      <c r="M27" s="7" t="inlineStr"/>
     </row>
     <row r="28" ht="65" customHeight="1">
       <c r="A28" s="4" t="n">
@@ -1501,19 +1858,31 @@
       </c>
       <c r="E28" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?player ?goals WHERE {
+  ?player p:P54 ?statement .
+  ?statement ps:P54 wd:Q42267 .
+  ?statement pq:P1351 ?goals .
+}
+ORDER BY DESC(xsd:decimal(?goals))
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F28" s="5" t="inlineStr"/>
+      <c r="G28" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F28" s="4" t="inlineStr">
+      <c r="H28" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00654.json</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr"/>
-      <c r="H28" s="5" t="inlineStr"/>
       <c r="I28" s="5" t="inlineStr"/>
       <c r="J28" s="5" t="inlineStr"/>
       <c r="K28" s="5" t="inlineStr"/>
+      <c r="L28" s="5" t="inlineStr"/>
+      <c r="M28" s="5" t="inlineStr"/>
     </row>
     <row r="29" ht="65" customHeight="1">
       <c r="A29" s="6" t="n">
@@ -1536,19 +1905,34 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?supermarket ?supermarketLabel ?revenue WHERE {
+  ?supermarket wdt:P31 / wdt:P279 * wd:Q18043413 .
+  ?supermarket wdt:P159 ?hq .
+  ?hq wdt:P17 wd:Q145 .
+  ?supermarket wdt:P2139 ?revenue .
+  ?supermarket rdfs:label ?supermarketLabel .
+  FILTER(lang(?supermarketLabel) = 'en')
+}
+ORDER BY DESC(?revenue)
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F29" s="7" t="inlineStr"/>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F29" s="6" t="inlineStr">
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00458.json</t>
         </is>
       </c>
-      <c r="G29" s="7" t="inlineStr"/>
-      <c r="H29" s="7" t="inlineStr"/>
       <c r="I29" s="7" t="inlineStr"/>
       <c r="J29" s="7" t="inlineStr"/>
       <c r="K29" s="7" t="inlineStr"/>
+      <c r="L29" s="7" t="inlineStr"/>
+      <c r="M29" s="7" t="inlineStr"/>
     </row>
     <row r="30" ht="65" customHeight="1">
       <c r="A30" s="4" t="n">
@@ -1571,19 +1955,31 @@
       </c>
       <c r="E30" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?country ?area WHERE {
+  wd:Q27496 wdt:P17 ?country .
+  ?country wdt:P31 wd:Q6256 .
+  ?country wdt:P2046 ?area .
+}
+ORDER BY DESC(xsd:float(?area))
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F30" s="5" t="inlineStr"/>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F30" s="4" t="inlineStr">
+      <c r="H30" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00469.json</t>
         </is>
       </c>
-      <c r="G30" s="5" t="inlineStr"/>
-      <c r="H30" s="5" t="inlineStr"/>
       <c r="I30" s="5" t="inlineStr"/>
       <c r="J30" s="5" t="inlineStr"/>
       <c r="K30" s="5" t="inlineStr"/>
+      <c r="L30" s="5" t="inlineStr"/>
+      <c r="M30" s="5" t="inlineStr"/>
     </row>
     <row r="31" ht="65" customHeight="1">
       <c r="A31" s="6" t="n">
@@ -1606,19 +2002,33 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?singer ?label WHERE {
+  wd:Q19863017 wdt:P161 ?singer .
+  ?singer wdt:P106 ?occupation .
+  ?occupation rdfs:label ?occLabel .
+  ?singer rdfs:label ?label .
+  FILTER(LANG(?label) = "en")
+  FILTER(LANG(?occLabel) = "en")
+  FILTER(REGEX(?occLabel , "singer" , "i"))
+}</t>
+        </is>
+      </c>
+      <c r="F31" s="7" t="inlineStr"/>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F31" s="6" t="inlineStr">
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00641.json</t>
         </is>
       </c>
-      <c r="G31" s="7" t="inlineStr"/>
-      <c r="H31" s="7" t="inlineStr"/>
       <c r="I31" s="7" t="inlineStr"/>
       <c r="J31" s="7" t="inlineStr"/>
       <c r="K31" s="7" t="inlineStr"/>
+      <c r="L31" s="7" t="inlineStr"/>
+      <c r="M31" s="7" t="inlineStr"/>
     </row>
     <row r="32" ht="65" customHeight="1">
       <c r="A32" s="4" t="n">
@@ -1641,19 +2051,27 @@
       </c>
       <c r="E32" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?director WHERE {
+  wd:Q103372692 wdt:P57 ?director .
+}</t>
+        </is>
+      </c>
+      <c r="F32" s="5" t="inlineStr"/>
+      <c r="G32" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F32" s="4" t="inlineStr">
+      <c r="H32" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00088.json</t>
         </is>
       </c>
-      <c r="G32" s="5" t="inlineStr"/>
-      <c r="H32" s="5" t="inlineStr"/>
       <c r="I32" s="5" t="inlineStr"/>
       <c r="J32" s="5" t="inlineStr"/>
       <c r="K32" s="5" t="inlineStr"/>
+      <c r="L32" s="5" t="inlineStr"/>
+      <c r="M32" s="5" t="inlineStr"/>
     </row>
     <row r="33" ht="65" customHeight="1">
       <c r="A33" s="6" t="n">
@@ -1676,19 +2094,39 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?film ?filmLabel ?publicationDate WHERE {
+  ?film rdfs:label ?label
+  FILTER(LANG(?label) = 'en' &amp;&amp; CONTAINS(?label , 'Terminator'))
+  .
+  ?film wdt:P31 wd:Q11424 .
+  ?film rdfs:label ?filmLabel
+  FILTER(LANG(?filmLabel) = 'en')
+  .
+  OPTIONAL {
+    ?film wdt:P577 ?publicationDate
+  }
+  .
+}
+ORDER BY DESC(?publicationDate)
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F33" s="7" t="inlineStr"/>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F33" s="6" t="inlineStr">
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00315.json</t>
         </is>
       </c>
-      <c r="G33" s="7" t="inlineStr"/>
-      <c r="H33" s="7" t="inlineStr"/>
       <c r="I33" s="7" t="inlineStr"/>
       <c r="J33" s="7" t="inlineStr"/>
       <c r="K33" s="7" t="inlineStr"/>
+      <c r="L33" s="7" t="inlineStr"/>
+      <c r="M33" s="7" t="inlineStr"/>
     </row>
     <row r="34" ht="65" customHeight="1">
       <c r="A34" s="4" t="n">
@@ -1711,19 +2149,27 @@
       </c>
       <c r="E34" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?releaseDate WHERE {
+  ?episode rdfs:label "Safe House" @en ; wdt:P179 wd:Q13417244 ; wdt:P577 ?releaseDate .
+}</t>
+        </is>
+      </c>
+      <c r="F34" s="5" t="inlineStr"/>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F34" s="4" t="inlineStr">
+      <c r="H34" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00518.json</t>
         </is>
       </c>
-      <c r="G34" s="5" t="inlineStr"/>
-      <c r="H34" s="5" t="inlineStr"/>
       <c r="I34" s="5" t="inlineStr"/>
       <c r="J34" s="5" t="inlineStr"/>
       <c r="K34" s="5" t="inlineStr"/>
+      <c r="L34" s="5" t="inlineStr"/>
+      <c r="M34" s="5" t="inlineStr"/>
     </row>
     <row r="35" ht="65" customHeight="1">
       <c r="A35" s="6" t="n">
@@ -1746,19 +2192,29 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?actor ?label WHERE {
+  wd:Q64768529 wdt:P161 ?actor .
+  ?actor rdfs:label ?label .
+  FILTER(LANG(?label) = 'en')
+}</t>
+        </is>
+      </c>
+      <c r="F35" s="7" t="inlineStr"/>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F35" s="6" t="inlineStr">
+      <c r="H35" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00165.json</t>
         </is>
       </c>
-      <c r="G35" s="7" t="inlineStr"/>
-      <c r="H35" s="7" t="inlineStr"/>
       <c r="I35" s="7" t="inlineStr"/>
       <c r="J35" s="7" t="inlineStr"/>
       <c r="K35" s="7" t="inlineStr"/>
+      <c r="L35" s="7" t="inlineStr"/>
+      <c r="M35" s="7" t="inlineStr"/>
     </row>
     <row r="36" ht="65" customHeight="1">
       <c r="A36" s="4" t="n">
@@ -1790,19 +2246,32 @@
       </c>
       <c r="E36" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?person ?personLabel WHERE {
+  ?person wdt:P31 wd:Q5 .
+  ?person wdt:P39 wd:Q24040821 .
+  OPTIONAL {
+    ?person rdfs:label ?personLabel
+    FILTER(lang(?personLabel) = "en")
+  }
+}</t>
+        </is>
+      </c>
+      <c r="F36" s="5" t="inlineStr"/>
+      <c r="G36" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in KG than in Table</t>
         </is>
       </c>
-      <c r="F36" s="4" t="inlineStr">
+      <c r="H36" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00814.json</t>
         </is>
       </c>
-      <c r="G36" s="5" t="inlineStr"/>
-      <c r="H36" s="5" t="inlineStr"/>
       <c r="I36" s="5" t="inlineStr"/>
       <c r="J36" s="5" t="inlineStr"/>
       <c r="K36" s="5" t="inlineStr"/>
+      <c r="L36" s="5" t="inlineStr"/>
+      <c r="M36" s="5" t="inlineStr"/>
     </row>
     <row r="37" ht="65" customHeight="1">
       <c r="A37" s="6" t="n">
@@ -1825,19 +2294,40 @@
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
+          <t>SELECT(SUM(?numRaces) AS ?total) WHERE {
+  {
+    SELECT ?season WHERE {
+      ?season wdt:P31 wd:Q171879 ; wdt:P1346 wd:Q9671 ; wdt:P585 ?time .
+    }
+    ORDER BY ASC(?time)
+    LIMIT 1
+  } UNION {
+    SELECT ?season WHERE {
+      ?season wdt:P31 wd:Q171879 ; wdt:P1346 wd:Q9671 ; wdt:P585 ?time .
+    }
+    ORDER BY DESC(?time)
+    LIMIT 1
+  }
+  ?season wdt:P1113 ?numRaces .
+}</t>
+        </is>
+      </c>
+      <c r="F37" s="7" t="inlineStr"/>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F37" s="6" t="inlineStr">
+      <c r="H37" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/Sportsreason_TANQ_complex/00194.json</t>
         </is>
       </c>
-      <c r="G37" s="7" t="inlineStr"/>
-      <c r="H37" s="7" t="inlineStr"/>
       <c r="I37" s="7" t="inlineStr"/>
       <c r="J37" s="7" t="inlineStr"/>
       <c r="K37" s="7" t="inlineStr"/>
+      <c r="L37" s="7" t="inlineStr"/>
+      <c r="M37" s="7" t="inlineStr"/>
     </row>
     <row r="38" ht="65" customHeight="1">
       <c r="A38" s="4" t="n">
@@ -1860,19 +2350,27 @@
       </c>
       <c r="E38" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?captain WHERE {
+  wd:Q79800 wdt:P634 ?captain
+}</t>
+        </is>
+      </c>
+      <c r="F38" s="5" t="inlineStr"/>
+      <c r="G38" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F38" s="4" t="inlineStr">
+      <c r="H38" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00058.json</t>
         </is>
       </c>
-      <c r="G38" s="5" t="inlineStr"/>
-      <c r="H38" s="5" t="inlineStr"/>
       <c r="I38" s="5" t="inlineStr"/>
       <c r="J38" s="5" t="inlineStr"/>
       <c r="K38" s="5" t="inlineStr"/>
+      <c r="L38" s="5" t="inlineStr"/>
+      <c r="M38" s="5" t="inlineStr"/>
     </row>
     <row r="39" ht="65" customHeight="1">
       <c r="A39" s="6" t="n">
@@ -1895,19 +2393,27 @@
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
+          <t>SELECT(COUNT(?edition) AS ?winCount) WHERE {
+  ?edition wdt:P361 wd:Q19323 ; wdt:P1346 wd:Q334526 .
+}</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr"/>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F39" s="6" t="inlineStr">
+      <c r="H39" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_infobox_complex/00008.json</t>
         </is>
       </c>
-      <c r="G39" s="7" t="inlineStr"/>
-      <c r="H39" s="7" t="inlineStr"/>
       <c r="I39" s="7" t="inlineStr"/>
       <c r="J39" s="7" t="inlineStr"/>
       <c r="K39" s="7" t="inlineStr"/>
+      <c r="L39" s="7" t="inlineStr"/>
+      <c r="M39" s="7" t="inlineStr"/>
     </row>
     <row r="40" ht="65" customHeight="1">
       <c r="A40" s="4" t="n">
@@ -1930,19 +2436,28 @@
       </c>
       <c r="E40" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?goals WHERE {
+  wd:Q357984 p:P54 ?statement .
+  ?statement ps:P54 wd:Q166776 ; pq:P1351 ?goals .
+}</t>
+        </is>
+      </c>
+      <c r="F40" s="5" t="inlineStr"/>
+      <c r="G40" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F40" s="4" t="inlineStr">
+      <c r="H40" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00124.json</t>
         </is>
       </c>
-      <c r="G40" s="5" t="inlineStr"/>
-      <c r="H40" s="5" t="inlineStr"/>
       <c r="I40" s="5" t="inlineStr"/>
       <c r="J40" s="5" t="inlineStr"/>
       <c r="K40" s="5" t="inlineStr"/>
+      <c r="L40" s="5" t="inlineStr"/>
+      <c r="M40" s="5" t="inlineStr"/>
     </row>
     <row r="41" ht="65" customHeight="1">
       <c r="A41" s="6" t="n">
@@ -1970,19 +2485,29 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?genre ?genreLabel WHERE {
+  wd:Q83287 wdt:P136 ?genre .
+  ?genre rdfs:label ?genreLabel .
+  FILTER(LANG(?genreLabel) = "en")
+}</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr"/>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F41" s="6" t="inlineStr">
+      <c r="H41" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00015.json</t>
         </is>
       </c>
-      <c r="G41" s="7" t="inlineStr"/>
-      <c r="H41" s="7" t="inlineStr"/>
       <c r="I41" s="7" t="inlineStr"/>
       <c r="J41" s="7" t="inlineStr"/>
       <c r="K41" s="7" t="inlineStr"/>
+      <c r="L41" s="7" t="inlineStr"/>
+      <c r="M41" s="7" t="inlineStr"/>
     </row>
     <row r="42" ht="65" customHeight="1">
       <c r="A42" s="4" t="n">
@@ -2014,19 +2539,30 @@
       </c>
       <c r="E42" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?calendar ?label WHERE {
+  ?calendar wdt:P31 wd:Q12132 .
+  ?calendar rdfs:label ?label .
+  FILTER(LANG(?label) = 'en')
+}
+LIMIT 10</t>
+        </is>
+      </c>
+      <c r="F42" s="5" t="inlineStr"/>
+      <c r="G42" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F42" s="4" t="inlineStr">
+      <c r="H42" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/Qampari_wikitables_simple/00073.json</t>
         </is>
       </c>
-      <c r="G42" s="5" t="inlineStr"/>
-      <c r="H42" s="5" t="inlineStr"/>
       <c r="I42" s="5" t="inlineStr"/>
       <c r="J42" s="5" t="inlineStr"/>
       <c r="K42" s="5" t="inlineStr"/>
+      <c r="L42" s="5" t="inlineStr"/>
+      <c r="M42" s="5" t="inlineStr"/>
     </row>
     <row r="43" ht="65" customHeight="1">
       <c r="A43" s="6" t="n">
@@ -2049,19 +2585,38 @@
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?partner ?partnerLabel WHERE {
+  wd:Q457761 p:P1327 ?statement .
+  ?statement ps:P1327 ?partner .
+  ?partner wdt:P31 wd:Q5 .
+  ?partner wdt:P21 wd:Q6581097 .
+  ?statement pq:P580 ?start .
+  ?statement pq:P582 ?end .
+  FILTER(xsd:date(?start) &lt;= "2010-12-31" ^^ xsd:date)
+  FILTER(xsd:date(?end) &gt;= "2010-01-01" ^^ xsd:date)
+  OPTIONAL {
+    ?partner rdfs:label ?partnerLabel .
+    FILTER(LANG(?partnerLabel) = "en")
+  }
+}</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr"/>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F43" s="6" t="inlineStr">
+      <c r="H43" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/OTT_QA_dev_complex/00077.json</t>
         </is>
       </c>
-      <c r="G43" s="7" t="inlineStr"/>
-      <c r="H43" s="7" t="inlineStr"/>
       <c r="I43" s="7" t="inlineStr"/>
       <c r="J43" s="7" t="inlineStr"/>
       <c r="K43" s="7" t="inlineStr"/>
+      <c r="L43" s="7" t="inlineStr"/>
+      <c r="M43" s="7" t="inlineStr"/>
     </row>
     <row r="44" ht="65" customHeight="1">
       <c r="A44" s="4" t="n">
@@ -2089,19 +2644,32 @@
       </c>
       <c r="E44" s="4" t="inlineStr">
         <is>
+          <t>SELECT DISTINCT ?project ?projectLabel WHERE {
+  ?exoplanet wdt:P31 wd:Q44559 .
+  ?exoplanet wdt:P65 ?project .
+  ?project rdfs:label ?projectLabel .
+  FILTER(LANG(?projectLabel) = "en")
+  FILTER(REGEX(?projectLabel , "(?i)project|search|survey"))
+}
+ORDER BY ?projectLabel</t>
+        </is>
+      </c>
+      <c r="F44" s="5" t="inlineStr"/>
+      <c r="G44" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F44" s="4" t="inlineStr">
+      <c r="H44" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/Qampari_wikitables_simple/00051.json</t>
         </is>
       </c>
-      <c r="G44" s="5" t="inlineStr"/>
-      <c r="H44" s="5" t="inlineStr"/>
       <c r="I44" s="5" t="inlineStr"/>
       <c r="J44" s="5" t="inlineStr"/>
       <c r="K44" s="5" t="inlineStr"/>
+      <c r="L44" s="5" t="inlineStr"/>
+      <c r="M44" s="5" t="inlineStr"/>
     </row>
     <row r="45" ht="65" customHeight="1">
       <c r="A45" s="6" t="n">
@@ -2124,19 +2692,30 @@
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
+          <t>SELECT(COUNT(DISTINCT ?olympics) AS ?count) WHERE {
+  ?athlete wdt:P1344 wd:Q2775602 .
+  ?athlete wdt:P1532 wd:Q43 .
+  ?athlete wdt:P1344 ?olympics .
+  ?olympics wdt:P31 wd:Q202125 .
+}</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr"/>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F45" s="6" t="inlineStr">
+      <c r="H45" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/OTT_QA_dev_complex/00241.json</t>
         </is>
       </c>
-      <c r="G45" s="7" t="inlineStr"/>
-      <c r="H45" s="7" t="inlineStr"/>
       <c r="I45" s="7" t="inlineStr"/>
       <c r="J45" s="7" t="inlineStr"/>
       <c r="K45" s="7" t="inlineStr"/>
+      <c r="L45" s="7" t="inlineStr"/>
+      <c r="M45" s="7" t="inlineStr"/>
     </row>
     <row r="46" ht="65" customHeight="1">
       <c r="A46" s="4" t="n">
@@ -2168,19 +2747,32 @@
       </c>
       <c r="E46" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?galaxy ?label WHERE {
+  ?galaxy wdt:P31 / wdt:P279 * wd:Q752374 .
+  OPTIONAL {
+    ?galaxy rdfs:label ?label .
+    FILTER(LANG(?label) = "en")
+  }
+  FILTER(bound(?label))
+}</t>
+        </is>
+      </c>
+      <c r="F46" s="5" t="inlineStr"/>
+      <c r="G46" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F46" s="4" t="inlineStr">
+      <c r="H46" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/Qampari_wikitables_simple/00004.json</t>
         </is>
       </c>
-      <c r="G46" s="5" t="inlineStr"/>
-      <c r="H46" s="5" t="inlineStr"/>
       <c r="I46" s="5" t="inlineStr"/>
       <c r="J46" s="5" t="inlineStr"/>
       <c r="K46" s="5" t="inlineStr"/>
+      <c r="L46" s="5" t="inlineStr"/>
+      <c r="M46" s="5" t="inlineStr"/>
     </row>
     <row r="47" ht="65" customHeight="1">
       <c r="A47" s="6" t="n">
@@ -2203,19 +2795,39 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
+          <t>SELECT(COUNT(DISTINCT ?game) AS ?count) WHERE {
+  {
+    ?game wdt:P361 wd:Q3511178 .
+    ?game wdt:P276 wd:Q49136 .
+    ?game wdt:P710 wd:Q213959 .
+  } UNION {
+    ?game wdt:P361 wd:Q14870260 .
+    ?game wdt:P276 wd:Q49136 .
+    ?game wdt:P710 wd:Q213959 .
+  } UNION {
+    ?game wdt:P361 wd:Q56692089 .
+    ?game wdt:P276 wd:Q49136 .
+    ?game wdt:P710 wd:Q213959 .
+  }
+}</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="inlineStr"/>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F47" s="6" t="inlineStr">
+      <c r="H47" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/Sportsreason_TANQ_complex/00054.json</t>
         </is>
       </c>
-      <c r="G47" s="7" t="inlineStr"/>
-      <c r="H47" s="7" t="inlineStr"/>
       <c r="I47" s="7" t="inlineStr"/>
       <c r="J47" s="7" t="inlineStr"/>
       <c r="K47" s="7" t="inlineStr"/>
+      <c r="L47" s="7" t="inlineStr"/>
+      <c r="M47" s="7" t="inlineStr"/>
     </row>
     <row r="48" ht="65" customHeight="1">
       <c r="A48" s="4" t="n">
@@ -2238,19 +2850,27 @@
       </c>
       <c r="E48" s="4" t="inlineStr">
         <is>
+          <t>SELECT(COUNT(?child) AS ?count) WHERE {
+  wd:Q1380505 wdt:P40 ?child
+}</t>
+        </is>
+      </c>
+      <c r="F48" s="5" t="inlineStr"/>
+      <c r="G48" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F48" s="4" t="inlineStr">
+      <c r="H48" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_infobox_complex/00101.json</t>
         </is>
       </c>
-      <c r="G48" s="5" t="inlineStr"/>
-      <c r="H48" s="5" t="inlineStr"/>
       <c r="I48" s="5" t="inlineStr"/>
       <c r="J48" s="5" t="inlineStr"/>
       <c r="K48" s="5" t="inlineStr"/>
+      <c r="L48" s="5" t="inlineStr"/>
+      <c r="M48" s="5" t="inlineStr"/>
     </row>
     <row r="49" ht="65" customHeight="1">
       <c r="A49" s="6" t="n">
@@ -2273,19 +2893,30 @@
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?awardLabel WHERE {
+  wd:Q483325 wdt:P166 ?award .
+  ?award rdfs:label ?awardLabel .
+  FILTER(LANG(?awardLabel) = "en")
+  FILTER(CONTAINS(LCASE(?awardLabel) , "annie") &amp;&amp; CONTAINS(LCASE(?awardLabel) , "voice"))
+}</t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="inlineStr"/>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F49" s="6" t="inlineStr">
+      <c r="H49" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00084.json</t>
         </is>
       </c>
-      <c r="G49" s="7" t="inlineStr"/>
-      <c r="H49" s="7" t="inlineStr"/>
       <c r="I49" s="7" t="inlineStr"/>
       <c r="J49" s="7" t="inlineStr"/>
       <c r="K49" s="7" t="inlineStr"/>
+      <c r="L49" s="7" t="inlineStr"/>
+      <c r="M49" s="7" t="inlineStr"/>
     </row>
     <row r="50" ht="65" customHeight="1">
       <c r="A50" s="4" t="n">
@@ -2308,19 +2939,33 @@
       </c>
       <c r="E50" s="4" t="inlineStr">
         <is>
+          <t>SELECT(SUM(xsd:integer(?wins) + xsd:integer(?losses)) AS ?totalGames) WHERE {
+  VALUES ?series {
+    wd:Q253000 wd:Q278844 wd:Q5145502
+  }
+  ?series p:P1532 ?participantStatement .
+  ?participantStatement ps:P1532 wd:Q166634 .
+  ?participantStatement pq:P5049 ?wins .
+  ?participantStatement pq:P5050 ?losses .
+}</t>
+        </is>
+      </c>
+      <c r="F50" s="5" t="inlineStr"/>
+      <c r="G50" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F50" s="4" t="inlineStr">
+      <c r="H50" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/Sportsreason_TANQ_complex/00147.json</t>
         </is>
       </c>
-      <c r="G50" s="5" t="inlineStr"/>
-      <c r="H50" s="5" t="inlineStr"/>
       <c r="I50" s="5" t="inlineStr"/>
       <c r="J50" s="5" t="inlineStr"/>
       <c r="K50" s="5" t="inlineStr"/>
+      <c r="L50" s="5" t="inlineStr"/>
+      <c r="M50" s="5" t="inlineStr"/>
     </row>
     <row r="51" ht="65" customHeight="1">
       <c r="A51" s="6" t="n">
@@ -2343,19 +2988,29 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?designer ?designerLabel WHERE {
+  wd:Q409022 wdt:P2554 ?designer .
+  ?designer rdfs:label ?designerLabel .
+  FILTER(LANG(?designerLabel) = 'en')
+}</t>
+        </is>
+      </c>
+      <c r="F51" s="7" t="inlineStr"/>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F51" s="6" t="inlineStr">
+      <c r="H51" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00104.json</t>
         </is>
       </c>
-      <c r="G51" s="7" t="inlineStr"/>
-      <c r="H51" s="7" t="inlineStr"/>
       <c r="I51" s="7" t="inlineStr"/>
       <c r="J51" s="7" t="inlineStr"/>
       <c r="K51" s="7" t="inlineStr"/>
+      <c r="L51" s="7" t="inlineStr"/>
+      <c r="M51" s="7" t="inlineStr"/>
     </row>
     <row r="52" ht="65" customHeight="1">
       <c r="A52" s="4" t="n">
@@ -2378,19 +3033,32 @@
       </c>
       <c r="E52" s="4" t="inlineStr">
         <is>
+          <t>SELECT(SUM(?numGames) AS ?totalGames) WHERE {
+  VALUES ?seriesLabel {
+    "1982 National League Championship Series" @en "2006 National League Championship Series" @en "2011 World Series" @en "2013 National League Championship Series" @en "2011 National League Championship Series" @en
+  }
+  ?series rdfs:label ?seriesLabel .
+  ?series wdt:P710 wd:Q166474 .
+  ?series wdt:P2633 ?numGames .
+}</t>
+        </is>
+      </c>
+      <c r="F52" s="5" t="inlineStr"/>
+      <c r="G52" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F52" s="4" t="inlineStr">
+      <c r="H52" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/Sportsreason_TANQ_complex/00004.json</t>
         </is>
       </c>
-      <c r="G52" s="5" t="inlineStr"/>
-      <c r="H52" s="5" t="inlineStr"/>
       <c r="I52" s="5" t="inlineStr"/>
       <c r="J52" s="5" t="inlineStr"/>
       <c r="K52" s="5" t="inlineStr"/>
+      <c r="L52" s="5" t="inlineStr"/>
+      <c r="M52" s="5" t="inlineStr"/>
     </row>
     <row r="53" ht="65" customHeight="1">
       <c r="A53" s="6" t="n">
@@ -2413,19 +3081,31 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
+          <t>SELECT(COUNT(?game) AS ?total) WHERE {
+  VALUES ?series {
+    wd:Q56692089 wd:Q14870260 wd:Q3511178
+  }
+  ?game wdt:P361 ?series .
+  ?game wdt:P276 wd:Q49136 .
+}</t>
+        </is>
+      </c>
+      <c r="F53" s="7" t="inlineStr"/>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F53" s="6" t="inlineStr">
+      <c r="H53" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/Sportsreason_TANQ_complex/00081.json</t>
         </is>
       </c>
-      <c r="G53" s="7" t="inlineStr"/>
-      <c r="H53" s="7" t="inlineStr"/>
       <c r="I53" s="7" t="inlineStr"/>
       <c r="J53" s="7" t="inlineStr"/>
       <c r="K53" s="7" t="inlineStr"/>
+      <c r="L53" s="7" t="inlineStr"/>
+      <c r="M53" s="7" t="inlineStr"/>
     </row>
     <row r="54" ht="65" customHeight="1">
       <c r="A54" s="4" t="n">
@@ -2448,19 +3128,31 @@
       </c>
       <c r="E54" s="4" t="inlineStr">
         <is>
+          <t>SELECT(SUM(?games) AS ?totalGames) WHERE {
+  VALUES ?year {
+    1977 1978 1983 2008 2009
+  }
+  ?season wdt:P31 wd:Q1987735 ; wdt:P179 wd:Q702315 ; wdt:P7232 wd:Q334634 ; wdt:P7232 wd:Q650840 ; wdt:P585 ?dateTime ; wdt:P8409 ?games .
+  FILTER(YEAR(?dateTime) = ?year)
+}</t>
+        </is>
+      </c>
+      <c r="F54" s="5" t="inlineStr"/>
+      <c r="G54" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F54" s="4" t="inlineStr">
+      <c r="H54" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/Sportsreason_TANQ_complex/00100.json</t>
         </is>
       </c>
-      <c r="G54" s="5" t="inlineStr"/>
-      <c r="H54" s="5" t="inlineStr"/>
       <c r="I54" s="5" t="inlineStr"/>
       <c r="J54" s="5" t="inlineStr"/>
       <c r="K54" s="5" t="inlineStr"/>
+      <c r="L54" s="5" t="inlineStr"/>
+      <c r="M54" s="5" t="inlineStr"/>
     </row>
     <row r="55" ht="65" customHeight="1">
       <c r="A55" s="6" t="n">
@@ -2483,19 +3175,33 @@
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?genre WHERE {
+  wd:Q105082070 schema:description ?desc .
+  FILTER(LANG(?desc) = "en")
+  .
+  FILTER(contains(?desc , "novel") || regex(?desc , "^(.* )?novel( .*)?$" , "i"))
+  .
+  BIND("novel" AS ?genre)
+  .
+}</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr"/>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F55" s="6" t="inlineStr">
+      <c r="H55" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00139.json</t>
         </is>
       </c>
-      <c r="G55" s="7" t="inlineStr"/>
-      <c r="H55" s="7" t="inlineStr"/>
       <c r="I55" s="7" t="inlineStr"/>
       <c r="J55" s="7" t="inlineStr"/>
       <c r="K55" s="7" t="inlineStr"/>
+      <c r="L55" s="7" t="inlineStr"/>
+      <c r="M55" s="7" t="inlineStr"/>
     </row>
     <row r="56" ht="65" customHeight="1">
       <c r="A56" s="4" t="n">
@@ -2518,19 +3224,31 @@
       </c>
       <c r="E56" s="4" t="inlineStr">
         <is>
+          <t>SELECT(COUNT(?game) AS ?count) WHERE {
+  VALUES ?series {
+    wd:Q3511178 wd:Q14870260 wd:Q56692089
+  }
+  ?game wdt:P361 ?series .
+  ?game wdt:P276 wd:Q49136 .
+}</t>
+        </is>
+      </c>
+      <c r="F56" s="5" t="inlineStr"/>
+      <c r="G56" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F56" s="4" t="inlineStr">
+      <c r="H56" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/Sportsreason_TANQ_complex/00182.json</t>
         </is>
       </c>
-      <c r="G56" s="5" t="inlineStr"/>
-      <c r="H56" s="5" t="inlineStr"/>
       <c r="I56" s="5" t="inlineStr"/>
       <c r="J56" s="5" t="inlineStr"/>
       <c r="K56" s="5" t="inlineStr"/>
+      <c r="L56" s="5" t="inlineStr"/>
+      <c r="M56" s="5" t="inlineStr"/>
     </row>
     <row r="57" ht="65" customHeight="1">
       <c r="A57" s="6" t="n">
@@ -2553,19 +3271,33 @@
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?team ?teamLabel WHERE {
+  wd:Q615 p:P54 ?statement .
+  ?statement ps:P54 ?team ; pq:P580 ?startDate .
+  ?team rdfs:label ?teamLabel .
+  FILTER(LANG(?teamLabel) = "en")
+  .
+}
+ORDER BY ASC(?startDate)
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr"/>
+      <c r="G57" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F57" s="6" t="inlineStr">
+      <c r="H57" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00172.json</t>
         </is>
       </c>
-      <c r="G57" s="7" t="inlineStr"/>
-      <c r="H57" s="7" t="inlineStr"/>
       <c r="I57" s="7" t="inlineStr"/>
       <c r="J57" s="7" t="inlineStr"/>
       <c r="K57" s="7" t="inlineStr"/>
+      <c r="L57" s="7" t="inlineStr"/>
+      <c r="M57" s="7" t="inlineStr"/>
     </row>
     <row r="58" ht="65" customHeight="1">
       <c r="A58" s="4" t="n">
@@ -2588,19 +3320,35 @@
       </c>
       <c r="E58" s="4" t="inlineStr">
         <is>
+          <t>SELECT(SUM(?numGames) AS ?total) WHERE {
+  VALUES ?year {
+    1977 1978 2008 2009
+  }
+  ?series wdt:P361 wd:Q190280 .
+  ?series wdt:P585 ?date .
+  ?series wdt:P710 wd:Q334634 .
+  ?series wdt:P710 wd:Q650840 .
+  ?series wdt:P4231 ?numGames .
+  FILTER(YEAR(?date) = ?year)
+}</t>
+        </is>
+      </c>
+      <c r="F58" s="5" t="inlineStr"/>
+      <c r="G58" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F58" s="4" t="inlineStr">
+      <c r="H58" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/Sportsreason_TANQ_complex/00120.json</t>
         </is>
       </c>
-      <c r="G58" s="5" t="inlineStr"/>
-      <c r="H58" s="5" t="inlineStr"/>
       <c r="I58" s="5" t="inlineStr"/>
       <c r="J58" s="5" t="inlineStr"/>
       <c r="K58" s="5" t="inlineStr"/>
+      <c r="L58" s="5" t="inlineStr"/>
+      <c r="M58" s="5" t="inlineStr"/>
     </row>
     <row r="59" ht="65" customHeight="1">
       <c r="A59" s="6" t="n">
@@ -2623,19 +3371,31 @@
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
+          <t>SELECT(SUM(?games) AS ?totalGames) WHERE {
+  VALUES ?year {
+    1977 1978 2008 2009
+  }
+  ?season wdt:P3450 wd:Q182085 ; wdt:P580 ?startTime ; wdt:P710 wd:Q334634 ; wdt:P710 wd:Q650840 ; wdt:P1350 ?games .
+  FILTER(YEAR(?startTime) = ?year)
+}</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr"/>
+      <c r="G59" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F59" s="6" t="inlineStr">
+      <c r="H59" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/Sportsreason_TANQ_complex/00135.json</t>
         </is>
       </c>
-      <c r="G59" s="7" t="inlineStr"/>
-      <c r="H59" s="7" t="inlineStr"/>
       <c r="I59" s="7" t="inlineStr"/>
       <c r="J59" s="7" t="inlineStr"/>
       <c r="K59" s="7" t="inlineStr"/>
+      <c r="L59" s="7" t="inlineStr"/>
+      <c r="M59" s="7" t="inlineStr"/>
     </row>
     <row r="60" ht="65" customHeight="1">
       <c r="A60" s="4" t="n">
@@ -2658,19 +3418,31 @@
       </c>
       <c r="E60" s="4" t="inlineStr">
         <is>
+          <t>SELECT(SUM(?goals) AS ?totalGoals) WHERE {
+  ?match wdt:P641 wd:Q93704 .
+  ?match wdt:P585 ?date .
+  FILTER(YEAR(?date) = 1971)
+  ?match p:P4511 ?goalStatement .
+  ?goalStatement ps:P4511 ?goals ; pq:P4518 wd:Q12897 .
+}</t>
+        </is>
+      </c>
+      <c r="F60" s="5" t="inlineStr"/>
+      <c r="G60" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F60" s="4" t="inlineStr">
+      <c r="H60" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_table_complex/00075.json</t>
         </is>
       </c>
-      <c r="G60" s="5" t="inlineStr"/>
-      <c r="H60" s="5" t="inlineStr"/>
       <c r="I60" s="5" t="inlineStr"/>
       <c r="J60" s="5" t="inlineStr"/>
       <c r="K60" s="5" t="inlineStr"/>
+      <c r="L60" s="5" t="inlineStr"/>
+      <c r="M60" s="5" t="inlineStr"/>
     </row>
     <row r="61" ht="65" customHeight="1">
       <c r="A61" s="6" t="n">
@@ -2694,19 +3466,35 @@
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
+          <t>SELECT DISTINCT ?team ?teamLabel WHERE {
+  ?player wdt:P413 wd:Q201330 .
+  ?player p:P1344 ?statement .
+  ?statement pq:P54 ?team .
+  ?statement pq:P1351 ?goals .
+  FILTER(xsd:integer(?goals) &gt; 0)
+  .
+  ?team rdfs:label ?teamLabel .
+  FILTER(LANG(?teamLabel) = 'en')
+  .
+}</t>
+        </is>
+      </c>
+      <c r="F61" s="7" t="inlineStr"/>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F61" s="6" t="inlineStr">
+      <c r="H61" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/Qampari_wikitables_simple/00022.json</t>
         </is>
       </c>
-      <c r="G61" s="7" t="inlineStr"/>
-      <c r="H61" s="7" t="inlineStr"/>
       <c r="I61" s="7" t="inlineStr"/>
       <c r="J61" s="7" t="inlineStr"/>
       <c r="K61" s="7" t="inlineStr"/>
+      <c r="L61" s="7" t="inlineStr"/>
+      <c r="M61" s="7" t="inlineStr"/>
     </row>
     <row r="62" ht="65" customHeight="1">
       <c r="A62" s="4" t="n">
@@ -2738,19 +3526,30 @@
       </c>
       <c r="E62" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?weapon ?label WHERE {
+  ?weapon wdt:P279 wd:Q1194268 .
+  ?weapon rdfs:label ?label .
+  FILTER(LANG(?label) = "en")
+}
+LIMIT 10</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr"/>
+      <c r="G62" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F62" s="4" t="inlineStr">
+      <c r="H62" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/Qampari_wikitables_simple/00009.json</t>
         </is>
       </c>
-      <c r="G62" s="5" t="inlineStr"/>
-      <c r="H62" s="5" t="inlineStr"/>
       <c r="I62" s="5" t="inlineStr"/>
       <c r="J62" s="5" t="inlineStr"/>
       <c r="K62" s="5" t="inlineStr"/>
+      <c r="L62" s="5" t="inlineStr"/>
+      <c r="M62" s="5" t="inlineStr"/>
     </row>
     <row r="63" ht="65" customHeight="1">
       <c r="A63" s="6" t="n">
@@ -2778,19 +3577,29 @@
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?weapon ?label WHERE {
+  ?weapon wdt:P279 wd:Q3753913 .
+  ?weapon rdfs:label ?label .
+  FILTER(LANG(?label) = "en")
+}</t>
+        </is>
+      </c>
+      <c r="F63" s="7" t="inlineStr"/>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F63" s="6" t="inlineStr">
+      <c r="H63" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/Qampari_wikitables_simple/00048.json</t>
         </is>
       </c>
-      <c r="G63" s="7" t="inlineStr"/>
-      <c r="H63" s="7" t="inlineStr"/>
       <c r="I63" s="7" t="inlineStr"/>
       <c r="J63" s="7" t="inlineStr"/>
       <c r="K63" s="7" t="inlineStr"/>
+      <c r="L63" s="7" t="inlineStr"/>
+      <c r="M63" s="7" t="inlineStr"/>
     </row>
     <row r="64" ht="65" customHeight="1">
       <c r="A64" s="4" t="n">
@@ -2813,19 +3622,27 @@
       </c>
       <c r="E64" s="4" t="inlineStr">
         <is>
+          <t>SELECT(COUNT(?member) AS ?count) WHERE {
+  wd:Q2511310 wdt:P527 ?member
+}</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr"/>
+      <c r="G64" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F64" s="4" t="inlineStr">
+      <c r="H64" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_infobox_complex/00298.json</t>
         </is>
       </c>
-      <c r="G64" s="5" t="inlineStr"/>
-      <c r="H64" s="5" t="inlineStr"/>
       <c r="I64" s="5" t="inlineStr"/>
       <c r="J64" s="5" t="inlineStr"/>
       <c r="K64" s="5" t="inlineStr"/>
+      <c r="L64" s="5" t="inlineStr"/>
+      <c r="M64" s="5" t="inlineStr"/>
     </row>
     <row r="65" ht="65" customHeight="1">
       <c r="A65" s="6" t="n">
@@ -2848,19 +3665,35 @@
       </c>
       <c r="E65" s="6" t="inlineStr">
         <is>
+          <t>SELECT(COUNT(?movie) AS ?count) WHERE {
+  ?movie wdt:P179 wd:Q2716420 .
+  ?movie wdt:P31 / wdt:P279 * wd:Q11424 .
+  ?movie rdfs:label ?title .
+  FILTER(LANG(?title) = 'en')
+  .
+  FILTER(CONTAINS(LCASE(?title) , "die hard"))
+  .
+  ?movie wdt:P577 ?releaseDate .
+  FILTER(xsd:dateTime(?releaseDate) &lt; "2013-01-01T00:00:00Z" ^^ xsd:dateTime)
+}</t>
+        </is>
+      </c>
+      <c r="F65" s="7" t="inlineStr"/>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F65" s="6" t="inlineStr">
+      <c r="H65" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_table_complex/00007.json</t>
         </is>
       </c>
-      <c r="G65" s="7" t="inlineStr"/>
-      <c r="H65" s="7" t="inlineStr"/>
       <c r="I65" s="7" t="inlineStr"/>
       <c r="J65" s="7" t="inlineStr"/>
       <c r="K65" s="7" t="inlineStr"/>
+      <c r="L65" s="7" t="inlineStr"/>
+      <c r="M65" s="7" t="inlineStr"/>
     </row>
     <row r="66" ht="65" customHeight="1">
       <c r="A66" s="4" t="n">
@@ -2883,19 +3716,27 @@
       </c>
       <c r="E66" s="4" t="inlineStr">
         <is>
+          <t>SELECT(COUNT(?province) AS ?count) WHERE {
+  ?province wdt:P31 wd:Q30566856 ; wdt:P17 wd:Q252
+}</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr"/>
+      <c r="G66" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F66" s="4" t="inlineStr">
+      <c r="H66" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/OTT_QA_dev_complex/00172.json</t>
         </is>
       </c>
-      <c r="G66" s="5" t="inlineStr"/>
-      <c r="H66" s="5" t="inlineStr"/>
       <c r="I66" s="5" t="inlineStr"/>
       <c r="J66" s="5" t="inlineStr"/>
       <c r="K66" s="5" t="inlineStr"/>
+      <c r="L66" s="5" t="inlineStr"/>
+      <c r="M66" s="5" t="inlineStr"/>
     </row>
     <row r="67" ht="65" customHeight="1">
       <c r="A67" s="6" t="n">
@@ -2918,19 +3759,29 @@
       </c>
       <c r="E67" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?hero ?heroLabel WHERE {
+  wd:Q4941 wdt:P674 ?hero .
+  ?hero rdfs:label ?heroLabel .
+  FILTER(LANG(?heroLabel) = "en")
+}</t>
+        </is>
+      </c>
+      <c r="F67" s="7" t="inlineStr"/>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F67" s="6" t="inlineStr">
+      <c r="H67" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00051.json</t>
         </is>
       </c>
-      <c r="G67" s="7" t="inlineStr"/>
-      <c r="H67" s="7" t="inlineStr"/>
       <c r="I67" s="7" t="inlineStr"/>
       <c r="J67" s="7" t="inlineStr"/>
       <c r="K67" s="7" t="inlineStr"/>
+      <c r="L67" s="7" t="inlineStr"/>
+      <c r="M67" s="7" t="inlineStr"/>
     </row>
     <row r="68" ht="65" customHeight="1">
       <c r="A68" s="4" t="n">
@@ -2953,19 +3804,32 @@
       </c>
       <c r="E68" s="4" t="inlineStr">
         <is>
+          <t>SELECT(COUNT(?larger) + 1 AS ?rank) WHERE {
+  wd:Q974 wdt:P2171 ?drcSize .
+  ?larger wdt:P2171 ?largerSize ; wdt:P31 wd:Q6256 ; wdt:P30 wd:Q15 .
+  FILTER(?larger != wd:Q974)
+  FILTER(xsd:integer(?largerSize) &gt; xsd:integer(?drcSize))
+  FILTER(ISNUMERIC(xsd:integer(?largerSize)))
+  FILTER(ISNUMERIC(xsd:integer(?drcSize)))
+}</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr"/>
+      <c r="G68" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F68" s="4" t="inlineStr">
+      <c r="H68" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/Monaco_time_complex/00029.json</t>
         </is>
       </c>
-      <c r="G68" s="5" t="inlineStr"/>
-      <c r="H68" s="5" t="inlineStr"/>
       <c r="I68" s="5" t="inlineStr"/>
       <c r="J68" s="5" t="inlineStr"/>
       <c r="K68" s="5" t="inlineStr"/>
+      <c r="L68" s="5" t="inlineStr"/>
+      <c r="M68" s="5" t="inlineStr"/>
     </row>
     <row r="69" ht="65" customHeight="1">
       <c r="A69" s="6" t="n">
@@ -2988,19 +3852,53 @@
       </c>
       <c r="E69" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?lakeLabel WHERE {
+  {
+    SELECT ?city WHERE {
+      ?city wdt:P17 wd:Q16 .
+      ?city wdt:P31 / wdt:P279 * wd:Q515 .
+      ?city p:P1082 ?popStmt .
+      ?popStmt ps:P1082 ?population ; pq:P585 ?time .
+      FILTER(isNumeric(?population))
+      {
+        SELECT ?city(MAX(?time) AS ?latestTime) WHERE {
+          ?city p:P1082 ?stmt .
+          ?stmt pq:P585 ?time .
+          FILTER(datatype(?time) = xsd:dateTime)
+        }
+        GROUP BY ?city
+      }
+      FILTER(?time = ?latestTime)
+    }
+    ORDER BY xsd:integer(?population)
+    LIMIT 1
+  }
+  ?city wdt:P625 ?cityCoord .
+  ?lake wdt:P31 wd:Q39715 ; wdt:P625 ?lakeCoord .
+  ?lake rdfs:label ?lakeLabel .
+  FILTER(lang(?lakeLabel) = 'en')
+  FILTER(geof:distance(?cityCoord , ?lakeCoord) &lt; 200000)
+}
+ORDER BY geof:distance(?cityCoord , ?lakeCoord)
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F69" s="7" t="inlineStr"/>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F69" s="6" t="inlineStr">
+      <c r="H69" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/OTT_QA_dev_complex/00337.json</t>
         </is>
       </c>
-      <c r="G69" s="7" t="inlineStr"/>
-      <c r="H69" s="7" t="inlineStr"/>
       <c r="I69" s="7" t="inlineStr"/>
       <c r="J69" s="7" t="inlineStr"/>
       <c r="K69" s="7" t="inlineStr"/>
+      <c r="L69" s="7" t="inlineStr"/>
+      <c r="M69" s="7" t="inlineStr"/>
     </row>
     <row r="70" ht="65" customHeight="1">
       <c r="A70" s="4" t="n">
@@ -3023,19 +3921,34 @@
       </c>
       <c r="E70" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?song ?label WHERE {
+  ?song wdt:P31 / wdt:P279 * wd:Q386724 .
+  ?song wdt:P577 ?date .
+  FILTER(YEAR(?date) = 2016)
+  .
+  ?song rdfs:label ?label .
+  FILTER(LANG(?label) = 'en')
+  .
+  FILTER(CONTAINS(LCASE(?label) , "start again"))
+}</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr"/>
+      <c r="G70" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F70" s="4" t="inlineStr">
+      <c r="H70" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/OTT_QA_dev_complex/00018.json</t>
         </is>
       </c>
-      <c r="G70" s="5" t="inlineStr"/>
-      <c r="H70" s="5" t="inlineStr"/>
       <c r="I70" s="5" t="inlineStr"/>
       <c r="J70" s="5" t="inlineStr"/>
       <c r="K70" s="5" t="inlineStr"/>
+      <c r="L70" s="5" t="inlineStr"/>
+      <c r="M70" s="5" t="inlineStr"/>
     </row>
     <row r="71" ht="65" customHeight="1">
       <c r="A71" s="6" t="n">
@@ -3058,19 +3971,31 @@
       </c>
       <c r="E71" s="6" t="inlineStr">
         <is>
+          <t>SELECT(COUNT(DISTINCT ?term) AS ?count) WHERE {
+  ?term ps:P39 wd:Q17324844 .
+  ?term pq:P4100 wd:Q10225 .
+  ?term pq:P768 wd:Q1363 .
+  ?term pq:P580 ?start .
+  FILTER(?start &gt;= "1952-01-01T00:00:00Z" ^^ xsd:dateTime)
+}</t>
+        </is>
+      </c>
+      <c r="F71" s="7" t="inlineStr"/>
+      <c r="G71" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F71" s="6" t="inlineStr">
+      <c r="H71" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/OTT_QA_dev_complex/00394.json</t>
         </is>
       </c>
-      <c r="G71" s="7" t="inlineStr"/>
-      <c r="H71" s="7" t="inlineStr"/>
       <c r="I71" s="7" t="inlineStr"/>
       <c r="J71" s="7" t="inlineStr"/>
       <c r="K71" s="7" t="inlineStr"/>
+      <c r="L71" s="7" t="inlineStr"/>
+      <c r="M71" s="7" t="inlineStr"/>
     </row>
     <row r="72" ht="65" customHeight="1">
       <c r="A72" s="4" t="n">
@@ -3093,19 +4018,28 @@
       </c>
       <c r="E72" s="4" t="inlineStr">
         <is>
+          <t>SELECT(COUNT(?race) AS ?count) WHERE {
+  ?race wdt:P31 wd:Q7965 ; wdt:P585 ?date ; wdt:P3764 wd:Q9673 .
+  FILTER(YEAR(?date) &gt;= 2016)
+}</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr"/>
+      <c r="G72" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F72" s="4" t="inlineStr">
+      <c r="H72" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/Sportsreason_TANQ_complex/00199.json</t>
         </is>
       </c>
-      <c r="G72" s="5" t="inlineStr"/>
-      <c r="H72" s="5" t="inlineStr"/>
       <c r="I72" s="5" t="inlineStr"/>
       <c r="J72" s="5" t="inlineStr"/>
       <c r="K72" s="5" t="inlineStr"/>
+      <c r="L72" s="5" t="inlineStr"/>
+      <c r="M72" s="5" t="inlineStr"/>
     </row>
     <row r="73" ht="65" customHeight="1">
       <c r="A73" s="6" t="n">
@@ -3128,19 +4062,29 @@
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
+          <t>SELECT(COUNT(*) AS ?count) WHERE {
+  ?season wdt:P1346 wd:Q620722 .
+  ?season rdfs:label ?label .
+  FILTER(CONTAINS(LCASE(?label) , "national challenge cup") &amp;&amp; LANG(?label) = "en")
+}</t>
+        </is>
+      </c>
+      <c r="F73" s="7" t="inlineStr"/>
+      <c r="G73" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F73" s="6" t="inlineStr">
+      <c r="H73" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_table_complex/00234.json</t>
         </is>
       </c>
-      <c r="G73" s="7" t="inlineStr"/>
-      <c r="H73" s="7" t="inlineStr"/>
       <c r="I73" s="7" t="inlineStr"/>
       <c r="J73" s="7" t="inlineStr"/>
       <c r="K73" s="7" t="inlineStr"/>
+      <c r="L73" s="7" t="inlineStr"/>
+      <c r="M73" s="7" t="inlineStr"/>
     </row>
     <row r="74" ht="65" customHeight="1">
       <c r="A74" s="4" t="n">
@@ -3163,19 +4107,27 @@
       </c>
       <c r="E74" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?owner WHERE {
+  wd:Q483020 wdt:P127 ?owner
+}</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr"/>
+      <c r="G74" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F74" s="4" t="inlineStr">
+      <c r="H74" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00323.json</t>
         </is>
       </c>
-      <c r="G74" s="5" t="inlineStr"/>
-      <c r="H74" s="5" t="inlineStr"/>
       <c r="I74" s="5" t="inlineStr"/>
       <c r="J74" s="5" t="inlineStr"/>
       <c r="K74" s="5" t="inlineStr"/>
+      <c r="L74" s="5" t="inlineStr"/>
+      <c r="M74" s="5" t="inlineStr"/>
     </row>
     <row r="75" ht="65" customHeight="1">
       <c r="A75" s="6" t="n">
@@ -3198,19 +4150,29 @@
       </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?actor ?actorLabel WHERE {
+  wd:Q56485183 wdt:P161 ?actor .
+  ?actor rdfs:label ?actorLabel .
+  FILTER(LANG(?actorLabel) = "en")
+}</t>
+        </is>
+      </c>
+      <c r="F75" s="7" t="inlineStr"/>
+      <c r="G75" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F75" s="6" t="inlineStr">
+      <c r="H75" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00031.json</t>
         </is>
       </c>
-      <c r="G75" s="7" t="inlineStr"/>
-      <c r="H75" s="7" t="inlineStr"/>
       <c r="I75" s="7" t="inlineStr"/>
       <c r="J75" s="7" t="inlineStr"/>
       <c r="K75" s="7" t="inlineStr"/>
+      <c r="L75" s="7" t="inlineStr"/>
+      <c r="M75" s="7" t="inlineStr"/>
     </row>
     <row r="76" ht="65" customHeight="1">
       <c r="A76" s="4" t="n">
@@ -3233,19 +4195,31 @@
       </c>
       <c r="E76" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?actor ?actorLabel WHERE {
+  wd:Q542866 wdt:P161 ?actor .
+  ?actor rdfs:label ?actorLabel .
+  FILTER(LANG(?actorLabel) = "en")
+  FILTER(CONTAINS(?actorLabel , "Pankaj Kapur"))
+}
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr"/>
+      <c r="G76" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F76" s="4" t="inlineStr">
+      <c r="H76" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00160.json</t>
         </is>
       </c>
-      <c r="G76" s="5" t="inlineStr"/>
-      <c r="H76" s="5" t="inlineStr"/>
       <c r="I76" s="5" t="inlineStr"/>
       <c r="J76" s="5" t="inlineStr"/>
       <c r="K76" s="5" t="inlineStr"/>
+      <c r="L76" s="5" t="inlineStr"/>
+      <c r="M76" s="5" t="inlineStr"/>
     </row>
     <row r="77" ht="65" customHeight="1">
       <c r="A77" s="6" t="n">
@@ -3268,19 +4242,27 @@
       </c>
       <c r="E77" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?date WHERE {
+  wd:Q542866 wdt:P577 ?date
+}</t>
+        </is>
+      </c>
+      <c r="F77" s="7" t="inlineStr"/>
+      <c r="G77" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F77" s="6" t="inlineStr">
+      <c r="H77" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_infobox_complex/00123.json</t>
         </is>
       </c>
-      <c r="G77" s="7" t="inlineStr"/>
-      <c r="H77" s="7" t="inlineStr"/>
       <c r="I77" s="7" t="inlineStr"/>
       <c r="J77" s="7" t="inlineStr"/>
       <c r="K77" s="7" t="inlineStr"/>
+      <c r="L77" s="7" t="inlineStr"/>
+      <c r="M77" s="7" t="inlineStr"/>
     </row>
     <row r="78" ht="65" customHeight="1">
       <c r="A78" s="4" t="n">
@@ -3303,19 +4285,28 @@
       </c>
       <c r="E78" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?dissolutionYear WHERE {
+  wd:Q11888530 wdt:P576 ?dissolution .
+  BIND(YEAR(?dissolution) AS ?dissolutionYear)
+}</t>
+        </is>
+      </c>
+      <c r="F78" s="5" t="inlineStr"/>
+      <c r="G78" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F78" s="4" t="inlineStr">
+      <c r="H78" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/OTT_QA_dev_complex/00283.json</t>
         </is>
       </c>
-      <c r="G78" s="5" t="inlineStr"/>
-      <c r="H78" s="5" t="inlineStr"/>
       <c r="I78" s="5" t="inlineStr"/>
       <c r="J78" s="5" t="inlineStr"/>
       <c r="K78" s="5" t="inlineStr"/>
+      <c r="L78" s="5" t="inlineStr"/>
+      <c r="M78" s="5" t="inlineStr"/>
     </row>
     <row r="79" ht="65" customHeight="1">
       <c r="A79" s="6" t="n">
@@ -3338,19 +4329,30 @@
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
+          <t>SELECT(YEAR(?birthDate) AS ?birthYear) WHERE {
+  ?member wdt:P463 wd:Q218837 .
+  ?member wdt:P569 ?birthDate .
+}
+ORDER BY ASC(?birthDate)
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F79" s="7" t="inlineStr"/>
+      <c r="G79" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F79" s="6" t="inlineStr">
+      <c r="H79" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/OTT_QA_dev_complex/00215.json</t>
         </is>
       </c>
-      <c r="G79" s="7" t="inlineStr"/>
-      <c r="H79" s="7" t="inlineStr"/>
       <c r="I79" s="7" t="inlineStr"/>
       <c r="J79" s="7" t="inlineStr"/>
       <c r="K79" s="7" t="inlineStr"/>
+      <c r="L79" s="7" t="inlineStr"/>
+      <c r="M79" s="7" t="inlineStr"/>
     </row>
     <row r="80" ht="65" customHeight="1">
       <c r="A80" s="4" t="n">
@@ -3373,19 +4375,29 @@
       </c>
       <c r="E80" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?coach ?coachLabel WHERE {
+  wd:Q78944434 wdt:P286 ?coach .
+  ?coach rdfs:label ?coachLabel .
+  FILTER(LANG(?coachLabel) = 'en')
+}</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr"/>
+      <c r="G80" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F80" s="4" t="inlineStr">
+      <c r="H80" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00121.json</t>
         </is>
       </c>
-      <c r="G80" s="5" t="inlineStr"/>
-      <c r="H80" s="5" t="inlineStr"/>
       <c r="I80" s="5" t="inlineStr"/>
       <c r="J80" s="5" t="inlineStr"/>
       <c r="K80" s="5" t="inlineStr"/>
+      <c r="L80" s="5" t="inlineStr"/>
+      <c r="M80" s="5" t="inlineStr"/>
     </row>
     <row r="81" ht="65" customHeight="1">
       <c r="A81" s="6" t="n">
@@ -3408,19 +4420,27 @@
       </c>
       <c r="E81" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?coach WHERE {
+  wd:Q16844931 wdt:P286 ?coach
+}</t>
+        </is>
+      </c>
+      <c r="F81" s="7" t="inlineStr"/>
+      <c r="G81" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F81" s="6" t="inlineStr">
+      <c r="H81" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00216.json</t>
         </is>
       </c>
-      <c r="G81" s="7" t="inlineStr"/>
-      <c r="H81" s="7" t="inlineStr"/>
       <c r="I81" s="7" t="inlineStr"/>
       <c r="J81" s="7" t="inlineStr"/>
       <c r="K81" s="7" t="inlineStr"/>
+      <c r="L81" s="7" t="inlineStr"/>
+      <c r="M81" s="7" t="inlineStr"/>
     </row>
     <row r="82" ht="65" customHeight="1">
       <c r="A82" s="4" t="n">
@@ -3445,19 +4465,31 @@
       </c>
       <c r="E82" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?author ?authorLabel WHERE {
+  wd:Q4417649 wdt:P50 ?author .
+  OPTIONAL {
+    ?author rdfs:label ?authorLabel .
+    FILTER(LANG(?authorLabel) = "en")
+  }
+}</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="inlineStr"/>
+      <c r="G82" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F82" s="4" t="inlineStr">
+      <c r="H82" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00190.json</t>
         </is>
       </c>
-      <c r="G82" s="5" t="inlineStr"/>
-      <c r="H82" s="5" t="inlineStr"/>
       <c r="I82" s="5" t="inlineStr"/>
       <c r="J82" s="5" t="inlineStr"/>
       <c r="K82" s="5" t="inlineStr"/>
+      <c r="L82" s="5" t="inlineStr"/>
+      <c r="M82" s="5" t="inlineStr"/>
     </row>
     <row r="83" ht="65" customHeight="1">
       <c r="A83" s="6" t="n">
@@ -3480,19 +4512,27 @@
       </c>
       <c r="E83" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?episodes WHERE {
+  wd:Q30322401 wdt:P1113 ?episodes .
+}</t>
+        </is>
+      </c>
+      <c r="F83" s="7" t="inlineStr"/>
+      <c r="G83" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F83" s="6" t="inlineStr">
+      <c r="H83" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00250.json</t>
         </is>
       </c>
-      <c r="G83" s="7" t="inlineStr"/>
-      <c r="H83" s="7" t="inlineStr"/>
       <c r="I83" s="7" t="inlineStr"/>
       <c r="J83" s="7" t="inlineStr"/>
       <c r="K83" s="7" t="inlineStr"/>
+      <c r="L83" s="7" t="inlineStr"/>
+      <c r="M83" s="7" t="inlineStr"/>
     </row>
     <row r="84" ht="65" customHeight="1">
       <c r="A84" s="4" t="n">
@@ -3515,19 +4555,29 @@
       </c>
       <c r="E84" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?date WHERE {
+  wd:Q24026109 wdt:P577 ?date .
+  wd:Q24026109 wdt:P495 wd:Q30 .
+}
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F84" s="5" t="inlineStr"/>
+      <c r="G84" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F84" s="4" t="inlineStr">
+      <c r="H84" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_table_complex/00048.json</t>
         </is>
       </c>
-      <c r="G84" s="5" t="inlineStr"/>
-      <c r="H84" s="5" t="inlineStr"/>
       <c r="I84" s="5" t="inlineStr"/>
       <c r="J84" s="5" t="inlineStr"/>
       <c r="K84" s="5" t="inlineStr"/>
+      <c r="L84" s="5" t="inlineStr"/>
+      <c r="M84" s="5" t="inlineStr"/>
     </row>
     <row r="85" ht="65" customHeight="1">
       <c r="A85" s="6" t="n">
@@ -3550,19 +4600,27 @@
       </c>
       <c r="E85" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?population WHERE {
+  wd:Q928 wdt:P1082 ?population .
+}</t>
+        </is>
+      </c>
+      <c r="F85" s="7" t="inlineStr"/>
+      <c r="G85" s="6" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F85" s="6" t="inlineStr">
+      <c r="H85" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/OTT_QA_dev_complex/00092.json</t>
         </is>
       </c>
-      <c r="G85" s="7" t="inlineStr"/>
-      <c r="H85" s="7" t="inlineStr"/>
       <c r="I85" s="7" t="inlineStr"/>
       <c r="J85" s="7" t="inlineStr"/>
       <c r="K85" s="7" t="inlineStr"/>
+      <c r="L85" s="7" t="inlineStr"/>
+      <c r="M85" s="7" t="inlineStr"/>
     </row>
     <row r="86" ht="65" customHeight="1">
       <c r="A86" s="4" t="n">
@@ -3585,19 +4643,28 @@
       </c>
       <c r="E86" s="4" t="inlineStr">
         <is>
+          <t>SELECT(YEAR(?date) AS ?year) WHERE {
+  wd:Q26505 wdt:P571 ?date
+}
+LIMIT 1</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr"/>
+      <c r="G86" s="4" t="inlineStr">
+        <is>
           <t>Different answer</t>
         </is>
       </c>
-      <c r="F86" s="4" t="inlineStr">
+      <c r="H86" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_table_complex/00266.json</t>
         </is>
       </c>
-      <c r="G86" s="5" t="inlineStr"/>
-      <c r="H86" s="5" t="inlineStr"/>
       <c r="I86" s="5" t="inlineStr"/>
       <c r="J86" s="5" t="inlineStr"/>
       <c r="K86" s="5" t="inlineStr"/>
+      <c r="L86" s="5" t="inlineStr"/>
+      <c r="M86" s="5" t="inlineStr"/>
     </row>
     <row r="87" ht="65" customHeight="1">
       <c r="A87" s="6" t="n">
@@ -3616,19 +4683,29 @@
       <c r="D87" s="6" t="inlineStr"/>
       <c r="E87" s="6" t="inlineStr">
         <is>
+          <t>SELECT(MAX(?age) AS ?maxAge) WHERE {
+  wd:Q340209 wdt:P569 ?birth ; wdt:P570 ?death .
+  BIND(YEAR(?death) - YEAR(?birth) AS ?age)
+  .
+}</t>
+        </is>
+      </c>
+      <c r="F87" s="7" t="inlineStr"/>
+      <c r="G87" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in Table than in KG</t>
         </is>
       </c>
-      <c r="F87" s="6" t="inlineStr">
+      <c r="H87" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/OTT_QA_dev_complex/00200.json</t>
         </is>
       </c>
-      <c r="G87" s="7" t="inlineStr"/>
-      <c r="H87" s="7" t="inlineStr"/>
       <c r="I87" s="7" t="inlineStr"/>
       <c r="J87" s="7" t="inlineStr"/>
       <c r="K87" s="7" t="inlineStr"/>
+      <c r="L87" s="7" t="inlineStr"/>
+      <c r="M87" s="7" t="inlineStr"/>
     </row>
     <row r="88" ht="65" customHeight="1">
       <c r="A88" s="4" t="n">
@@ -3651,19 +4728,29 @@
       </c>
       <c r="E88" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?owner ?ownerLabel WHERE {
+  wd:Q18729 wdt:P127 ?owner .
+  ?owner rdfs:label ?ownerLabel .
+  FILTER(LANG(?ownerLabel) = 'en')
+}</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr"/>
+      <c r="G88" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in Table than in KG</t>
         </is>
       </c>
-      <c r="F88" s="4" t="inlineStr">
+      <c r="H88" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00067.json</t>
         </is>
       </c>
-      <c r="G88" s="5" t="inlineStr"/>
-      <c r="H88" s="5" t="inlineStr"/>
       <c r="I88" s="5" t="inlineStr"/>
       <c r="J88" s="5" t="inlineStr"/>
       <c r="K88" s="5" t="inlineStr"/>
+      <c r="L88" s="5" t="inlineStr"/>
+      <c r="M88" s="5" t="inlineStr"/>
     </row>
     <row r="89" ht="65" customHeight="1">
       <c r="A89" s="6" t="n">
@@ -3686,19 +4773,30 @@
       </c>
       <c r="E89" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?countryLabel WHERE {
+  wd:Q2691159 wdt:P407 / wdt:P17 wd:Q145 .
+  wd:Q145 wdt:P150 ?subCountry .
+  ?subCountry rdfs:label ?countryLabel .
+  FILTER(LANG(?countryLabel) = 'en' &amp;&amp; CONTAINS(?countryLabel , 'England'))
+}</t>
+        </is>
+      </c>
+      <c r="F89" s="7" t="inlineStr"/>
+      <c r="G89" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in Table than in KG</t>
         </is>
       </c>
-      <c r="F89" s="6" t="inlineStr">
+      <c r="H89" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00179.json</t>
         </is>
       </c>
-      <c r="G89" s="7" t="inlineStr"/>
-      <c r="H89" s="7" t="inlineStr"/>
       <c r="I89" s="7" t="inlineStr"/>
       <c r="J89" s="7" t="inlineStr"/>
       <c r="K89" s="7" t="inlineStr"/>
+      <c r="L89" s="7" t="inlineStr"/>
+      <c r="M89" s="7" t="inlineStr"/>
     </row>
     <row r="90" ht="65" customHeight="1">
       <c r="A90" s="4" t="n">
@@ -3729,19 +4827,32 @@
       </c>
       <c r="E90" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?hotel ?label ?rooms WHERE {
+  ?hotel wdt:P31 wd:Q27686 .
+  ?hotel wdt:P8733 ?rooms .
+  FILTER(?rooms &gt;= 2000)
+  .
+  ?hotel rdfs:label ?label .
+  FILTER(LANG(?label) = "en")
+}</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr"/>
+      <c r="G90" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in Table than in KG</t>
         </is>
       </c>
-      <c r="F90" s="4" t="inlineStr">
+      <c r="H90" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/Qampari_wikitables_simple/00068.json</t>
         </is>
       </c>
-      <c r="G90" s="5" t="inlineStr"/>
-      <c r="H90" s="5" t="inlineStr"/>
       <c r="I90" s="5" t="inlineStr"/>
       <c r="J90" s="5" t="inlineStr"/>
       <c r="K90" s="5" t="inlineStr"/>
+      <c r="L90" s="5" t="inlineStr"/>
+      <c r="M90" s="5" t="inlineStr"/>
     </row>
     <row r="91" ht="65" customHeight="1">
       <c r="A91" s="6" t="n">
@@ -3764,19 +4875,33 @@
       </c>
       <c r="E91" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?actor ?actorLabel WHERE {
+  wd:Q62665 wdt:P161 ?actor .
+  VALUES ?actor {
+    wd:Q321 wd:Q59215
+  }
+  ?actor rdfs:label ?actorLabel .
+  FILTER(LANG(?actorLabel) = 'en')
+  .
+}</t>
+        </is>
+      </c>
+      <c r="F91" s="7" t="inlineStr"/>
+      <c r="G91" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in Table than in KG</t>
         </is>
       </c>
-      <c r="F91" s="6" t="inlineStr">
+      <c r="H91" s="6" t="inlineStr">
         <is>
           <t>ComplexQA/CompMix_infobox_complex/00005.json</t>
         </is>
       </c>
-      <c r="G91" s="7" t="inlineStr"/>
-      <c r="H91" s="7" t="inlineStr"/>
       <c r="I91" s="7" t="inlineStr"/>
       <c r="J91" s="7" t="inlineStr"/>
       <c r="K91" s="7" t="inlineStr"/>
+      <c r="L91" s="7" t="inlineStr"/>
+      <c r="M91" s="7" t="inlineStr"/>
     </row>
     <row r="92" ht="65" customHeight="1">
       <c r="A92" s="4" t="n">
@@ -3799,19 +4924,27 @@
       </c>
       <c r="E92" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?date WHERE {
+  wd:Q1573223 wdt:P577 ?date
+}</t>
+        </is>
+      </c>
+      <c r="F92" s="5" t="inlineStr"/>
+      <c r="G92" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in Table than in KG</t>
         </is>
       </c>
-      <c r="F92" s="4" t="inlineStr">
+      <c r="H92" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00779.json</t>
         </is>
       </c>
-      <c r="G92" s="5" t="inlineStr"/>
-      <c r="H92" s="5" t="inlineStr"/>
       <c r="I92" s="5" t="inlineStr"/>
       <c r="J92" s="5" t="inlineStr"/>
       <c r="K92" s="5" t="inlineStr"/>
+      <c r="L92" s="5" t="inlineStr"/>
+      <c r="M92" s="5" t="inlineStr"/>
     </row>
     <row r="93" ht="65" customHeight="1">
       <c r="A93" s="6" t="n">
@@ -3834,19 +4967,31 @@
       </c>
       <c r="E93" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?producer ?producerLabel WHERE {
+  wd:Q48672822 wdt:P162 ?producer .
+  OPTIONAL {
+    ?producer rdfs:label ?producerLabel
+    FILTER(lang(?producerLabel) = "en")
+  }
+}</t>
+        </is>
+      </c>
+      <c r="F93" s="7" t="inlineStr"/>
+      <c r="G93" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in Table than in KG</t>
         </is>
       </c>
-      <c r="F93" s="6" t="inlineStr">
+      <c r="H93" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00454.json</t>
         </is>
       </c>
-      <c r="G93" s="7" t="inlineStr"/>
-      <c r="H93" s="7" t="inlineStr"/>
       <c r="I93" s="7" t="inlineStr"/>
       <c r="J93" s="7" t="inlineStr"/>
       <c r="K93" s="7" t="inlineStr"/>
+      <c r="L93" s="7" t="inlineStr"/>
+      <c r="M93" s="7" t="inlineStr"/>
     </row>
     <row r="94" ht="65" customHeight="1">
       <c r="A94" s="4" t="n">
@@ -3869,19 +5014,29 @@
       </c>
       <c r="E94" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?genre ?genreLabel WHERE {
+  wd:Q944632 wdt:P136 ?genre .
+  ?genre rdfs:label ?genreLabel .
+  FILTER(LANG(?genreLabel) = "en")
+}</t>
+        </is>
+      </c>
+      <c r="F94" s="5" t="inlineStr"/>
+      <c r="G94" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in Table than in KG</t>
         </is>
       </c>
-      <c r="F94" s="4" t="inlineStr">
+      <c r="H94" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00486.json</t>
         </is>
       </c>
-      <c r="G94" s="5" t="inlineStr"/>
-      <c r="H94" s="5" t="inlineStr"/>
       <c r="I94" s="5" t="inlineStr"/>
       <c r="J94" s="5" t="inlineStr"/>
       <c r="K94" s="5" t="inlineStr"/>
+      <c r="L94" s="5" t="inlineStr"/>
+      <c r="M94" s="5" t="inlineStr"/>
     </row>
     <row r="95" ht="65" customHeight="1">
       <c r="A95" s="6" t="n">
@@ -3904,19 +5059,29 @@
       </c>
       <c r="E95" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?producer ?producerLabel WHERE {
+  wd:Q107597380 wdt:P162 ?producer .
+  ?producer rdfs:label ?producerLabel .
+  FILTER(LANG(?producerLabel) = 'en')
+}</t>
+        </is>
+      </c>
+      <c r="F95" s="7" t="inlineStr"/>
+      <c r="G95" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in Table than in KG</t>
         </is>
       </c>
-      <c r="F95" s="6" t="inlineStr">
+      <c r="H95" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00209.json</t>
         </is>
       </c>
-      <c r="G95" s="7" t="inlineStr"/>
-      <c r="H95" s="7" t="inlineStr"/>
       <c r="I95" s="7" t="inlineStr"/>
       <c r="J95" s="7" t="inlineStr"/>
       <c r="K95" s="7" t="inlineStr"/>
+      <c r="L95" s="7" t="inlineStr"/>
+      <c r="M95" s="7" t="inlineStr"/>
     </row>
     <row r="96" ht="65" customHeight="1">
       <c r="A96" s="4" t="n">
@@ -3935,19 +5100,30 @@
       <c r="D96" s="4" t="inlineStr"/>
       <c r="E96" s="4" t="inlineStr">
         <is>
+          <t>SELECT(MIN(YEAR(?collDate)) AS ?firstCollYear) WHERE {
+  VALUES ?collLeague {
+    wd:Q2352741 wd:Q50783
+  }
+  ?collSeason wdt:P118 ?collLeague ; wdt:P1346 wd:Q249679 ; wdt:P585 ?collDate .
+}</t>
+        </is>
+      </c>
+      <c r="F96" s="5" t="inlineStr"/>
+      <c r="G96" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in Table than in KG</t>
         </is>
       </c>
-      <c r="F96" s="4" t="inlineStr">
+      <c r="H96" s="4" t="inlineStr">
         <is>
           <t>ComplexQA/Sportsreason_TANQ_complex/00179.json</t>
         </is>
       </c>
-      <c r="G96" s="5" t="inlineStr"/>
-      <c r="H96" s="5" t="inlineStr"/>
       <c r="I96" s="5" t="inlineStr"/>
       <c r="J96" s="5" t="inlineStr"/>
       <c r="K96" s="5" t="inlineStr"/>
+      <c r="L96" s="5" t="inlineStr"/>
+      <c r="M96" s="5" t="inlineStr"/>
     </row>
     <row r="97" ht="65" customHeight="1">
       <c r="A97" s="6" t="n">
@@ -3978,19 +5154,34 @@
       </c>
       <c r="E97" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?characterName ?actor ?actorLabel WHERE {
+  wd:Q85518571 p:P725 ?statement .
+  ?statement ps:P725 ?actor .
+  ?statement pq:P453 ?characterName .
+  OPTIONAL {
+    ?actor rdfs:label ?actorLabel .
+    FILTER(lang(?actorLabel) = 'en')
+    .
+  }
+}</t>
+        </is>
+      </c>
+      <c r="F97" s="7" t="inlineStr"/>
+      <c r="G97" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in Table than in KG</t>
         </is>
       </c>
-      <c r="F97" s="6" t="inlineStr">
+      <c r="H97" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00119.json</t>
         </is>
       </c>
-      <c r="G97" s="7" t="inlineStr"/>
-      <c r="H97" s="7" t="inlineStr"/>
       <c r="I97" s="7" t="inlineStr"/>
       <c r="J97" s="7" t="inlineStr"/>
       <c r="K97" s="7" t="inlineStr"/>
+      <c r="L97" s="7" t="inlineStr"/>
+      <c r="M97" s="7" t="inlineStr"/>
     </row>
     <row r="98" ht="65" customHeight="1">
       <c r="A98" s="4" t="n">
@@ -4013,19 +5204,27 @@
       </c>
       <c r="E98" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?composer WHERE {
+  wd:Q20899576 wdt:P86 ?composer
+}</t>
+        </is>
+      </c>
+      <c r="F98" s="5" t="inlineStr"/>
+      <c r="G98" s="4" t="inlineStr">
+        <is>
           <t>Higher accuracy in Table than in KG</t>
         </is>
       </c>
-      <c r="F98" s="4" t="inlineStr">
+      <c r="H98" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00547.json</t>
         </is>
       </c>
-      <c r="G98" s="5" t="inlineStr"/>
-      <c r="H98" s="5" t="inlineStr"/>
       <c r="I98" s="5" t="inlineStr"/>
       <c r="J98" s="5" t="inlineStr"/>
       <c r="K98" s="5" t="inlineStr"/>
+      <c r="L98" s="5" t="inlineStr"/>
+      <c r="M98" s="5" t="inlineStr"/>
     </row>
     <row r="99" ht="65" customHeight="1">
       <c r="A99" s="6" t="n">
@@ -4048,19 +5247,29 @@
       </c>
       <c r="E99" s="6" t="inlineStr">
         <is>
+          <t>SELECT ?writer ?label WHERE {
+  wd:Q2881392 wdt:P676 ?writer .
+  ?writer rdfs:label ?label .
+  FILTER(lang(?label) = 'en')
+}</t>
+        </is>
+      </c>
+      <c r="F99" s="7" t="inlineStr"/>
+      <c r="G99" s="6" t="inlineStr">
+        <is>
           <t>Higher accuracy in Table than in KG</t>
         </is>
       </c>
-      <c r="F99" s="6" t="inlineStr">
+      <c r="H99" s="6" t="inlineStr">
         <is>
           <t>SimpleQA/NQ_table_test_simple/00623.json</t>
         </is>
       </c>
-      <c r="G99" s="7" t="inlineStr"/>
-      <c r="H99" s="7" t="inlineStr"/>
       <c r="I99" s="7" t="inlineStr"/>
       <c r="J99" s="7" t="inlineStr"/>
       <c r="K99" s="7" t="inlineStr"/>
+      <c r="L99" s="7" t="inlineStr"/>
+      <c r="M99" s="7" t="inlineStr"/>
     </row>
     <row r="100" ht="65" customHeight="1">
       <c r="A100" s="4" t="n">
@@ -4084,27 +5293,41 @@
       </c>
       <c r="E100" s="4" t="inlineStr">
         <is>
+          <t>SELECT ?team ?teamLabel WHERE {
+  wd:Q21621995 p:P54 ?statement .
+  ?statement ps:P54 ?team .
+  FILTER NOT EXISTS {
+    ?statement pq:P582 ?endTime
+  }
+  ?team rdfs:label ?teamLabel .
+  FILTER(LANG(?teamLabel) = "en")
+}</t>
+        </is>
+      </c>
+      <c r="F100" s="5" t="inlineStr"/>
+      <c r="G100" s="4" t="inlineStr">
+        <is>
           <t>Temporal changes</t>
         </is>
       </c>
-      <c r="F100" s="4" t="inlineStr">
+      <c r="H100" s="4" t="inlineStr">
         <is>
           <t>SimpleQA/CompMix_table_simple_qa/00055.json</t>
         </is>
       </c>
-      <c r="G100" s="5" t="inlineStr"/>
-      <c r="H100" s="5" t="inlineStr"/>
       <c r="I100" s="5" t="inlineStr"/>
       <c r="J100" s="5" t="inlineStr"/>
       <c r="K100" s="5" t="inlineStr"/>
+      <c r="L100" s="5" t="inlineStr"/>
+      <c r="M100" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K100"/>
+  <autoFilter ref="A1:M100"/>
   <dataValidations count="2">
-    <dataValidation sqref="G2:G100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Correct,Incorrect,Unsure"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H100 I2:I100 J2:J100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J100 K2:K100 L2:L100" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>